<commit_message>
Deploying to gh-pages from @ tarun2184/DEVLINK@7e85bd90bf3179924d99634922a9fc3c09a26cb9 🚀
</commit_message>
<xml_diff>
--- a/reports/Mobile_Appium_E2E_Test_Report_400.xlsx
+++ b/reports/Mobile_Appium_E2E_Test_Report_400.xlsx
@@ -52,7 +52,7 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-07T15:03:11.343Z</t>
+    <t>2026-08-07T15:22:43.166Z</t>
   </si>
   <si>
     <t>Verified Android Activity lifecycle and Capacitor native plugin interface</t>
@@ -3001,7 +3001,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
@@ -3027,7 +3027,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="4">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>12</v>
@@ -3053,7 +3053,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>12</v>
@@ -3079,7 +3079,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="4">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>12</v>
@@ -3105,7 +3105,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>12</v>
@@ -3131,7 +3131,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="4">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>12</v>
@@ -3157,7 +3157,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>12</v>
@@ -3183,7 +3183,7 @@
         <v>11</v>
       </c>
       <c r="E9" s="4">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>12</v>
@@ -3209,7 +3209,7 @@
         <v>11</v>
       </c>
       <c r="E10" s="2">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>12</v>
@@ -3235,7 +3235,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="4">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>12</v>
@@ -3261,7 +3261,7 @@
         <v>11</v>
       </c>
       <c r="E12" s="2">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>12</v>
@@ -3287,7 +3287,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="4">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>12</v>
@@ -3313,7 +3313,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>12</v>
@@ -3339,7 +3339,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="4">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>12</v>
@@ -3365,7 +3365,7 @@
         <v>11</v>
       </c>
       <c r="E16" s="2">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>12</v>
@@ -3391,7 +3391,7 @@
         <v>11</v>
       </c>
       <c r="E17" s="4">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>12</v>
@@ -3417,7 +3417,7 @@
         <v>11</v>
       </c>
       <c r="E18" s="2">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>12</v>
@@ -3443,7 +3443,7 @@
         <v>11</v>
       </c>
       <c r="E19" s="4">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>12</v>
@@ -3469,7 +3469,7 @@
         <v>11</v>
       </c>
       <c r="E20" s="2">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>12</v>
@@ -3495,7 +3495,7 @@
         <v>11</v>
       </c>
       <c r="E21" s="4">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>12</v>
@@ -3521,7 +3521,7 @@
         <v>11</v>
       </c>
       <c r="E22" s="2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>12</v>
@@ -3547,7 +3547,7 @@
         <v>11</v>
       </c>
       <c r="E23" s="4">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>12</v>
@@ -3573,7 +3573,7 @@
         <v>11</v>
       </c>
       <c r="E24" s="2">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>12</v>
@@ -3599,7 +3599,7 @@
         <v>11</v>
       </c>
       <c r="E25" s="4">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>12</v>
@@ -3625,7 +3625,7 @@
         <v>11</v>
       </c>
       <c r="E26" s="2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>12</v>
@@ -3651,7 +3651,7 @@
         <v>11</v>
       </c>
       <c r="E27" s="4">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>12</v>
@@ -3677,7 +3677,7 @@
         <v>11</v>
       </c>
       <c r="E28" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>12</v>
@@ -3703,7 +3703,7 @@
         <v>11</v>
       </c>
       <c r="E29" s="4">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>12</v>
@@ -3729,7 +3729,7 @@
         <v>11</v>
       </c>
       <c r="E30" s="2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>12</v>
@@ -3755,7 +3755,7 @@
         <v>11</v>
       </c>
       <c r="E31" s="4">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>12</v>
@@ -3781,7 +3781,7 @@
         <v>11</v>
       </c>
       <c r="E32" s="2">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>12</v>
@@ -3807,7 +3807,7 @@
         <v>11</v>
       </c>
       <c r="E33" s="4">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>12</v>
@@ -3833,7 +3833,7 @@
         <v>11</v>
       </c>
       <c r="E34" s="2">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
@@ -3859,7 +3859,7 @@
         <v>11</v>
       </c>
       <c r="E35" s="4">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>12</v>
@@ -3885,7 +3885,7 @@
         <v>11</v>
       </c>
       <c r="E36" s="2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
@@ -3911,7 +3911,7 @@
         <v>11</v>
       </c>
       <c r="E37" s="4">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>12</v>
@@ -3937,7 +3937,7 @@
         <v>11</v>
       </c>
       <c r="E38" s="2">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>12</v>
@@ -3963,7 +3963,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="4">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>12</v>
@@ -3989,7 +3989,7 @@
         <v>11</v>
       </c>
       <c r="E40" s="2">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>12</v>
@@ -4015,7 +4015,7 @@
         <v>11</v>
       </c>
       <c r="E41" s="4">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>12</v>
@@ -4041,7 +4041,7 @@
         <v>11</v>
       </c>
       <c r="E42" s="2">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>12</v>
@@ -4067,7 +4067,7 @@
         <v>11</v>
       </c>
       <c r="E43" s="4">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>12</v>
@@ -4093,7 +4093,7 @@
         <v>11</v>
       </c>
       <c r="E44" s="2">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>12</v>
@@ -4119,7 +4119,7 @@
         <v>11</v>
       </c>
       <c r="E45" s="4">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>12</v>
@@ -4145,7 +4145,7 @@
         <v>11</v>
       </c>
       <c r="E46" s="2">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>12</v>
@@ -4171,7 +4171,7 @@
         <v>11</v>
       </c>
       <c r="E47" s="4">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>12</v>
@@ -4197,7 +4197,7 @@
         <v>11</v>
       </c>
       <c r="E48" s="2">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>12</v>
@@ -4223,7 +4223,7 @@
         <v>11</v>
       </c>
       <c r="E49" s="4">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>12</v>
@@ -4249,7 +4249,7 @@
         <v>11</v>
       </c>
       <c r="E50" s="2">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>12</v>
@@ -4275,7 +4275,7 @@
         <v>11</v>
       </c>
       <c r="E51" s="4">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>12</v>
@@ -4301,7 +4301,7 @@
         <v>11</v>
       </c>
       <c r="E52" s="2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>12</v>
@@ -4327,7 +4327,7 @@
         <v>11</v>
       </c>
       <c r="E53" s="4">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>12</v>
@@ -4353,7 +4353,7 @@
         <v>11</v>
       </c>
       <c r="E54" s="2">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>12</v>
@@ -4379,7 +4379,7 @@
         <v>11</v>
       </c>
       <c r="E55" s="4">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>12</v>
@@ -4405,7 +4405,7 @@
         <v>11</v>
       </c>
       <c r="E56" s="2">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>12</v>
@@ -4431,7 +4431,7 @@
         <v>11</v>
       </c>
       <c r="E57" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>12</v>
@@ -4457,7 +4457,7 @@
         <v>11</v>
       </c>
       <c r="E58" s="2">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
@@ -4483,7 +4483,7 @@
         <v>11</v>
       </c>
       <c r="E59" s="4">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>12</v>
@@ -4509,7 +4509,7 @@
         <v>11</v>
       </c>
       <c r="E60" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>12</v>
@@ -4535,7 +4535,7 @@
         <v>11</v>
       </c>
       <c r="E61" s="4">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>12</v>
@@ -4561,7 +4561,7 @@
         <v>11</v>
       </c>
       <c r="E62" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>12</v>
@@ -4587,7 +4587,7 @@
         <v>11</v>
       </c>
       <c r="E63" s="4">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>12</v>
@@ -4613,7 +4613,7 @@
         <v>11</v>
       </c>
       <c r="E64" s="2">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>12</v>
@@ -4639,7 +4639,7 @@
         <v>11</v>
       </c>
       <c r="E65" s="4">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>12</v>
@@ -4665,7 +4665,7 @@
         <v>11</v>
       </c>
       <c r="E66" s="2">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>12</v>
@@ -4717,7 +4717,7 @@
         <v>11</v>
       </c>
       <c r="E68" s="2">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F68" s="3" t="s">
         <v>12</v>
@@ -4743,7 +4743,7 @@
         <v>11</v>
       </c>
       <c r="E69" s="4">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>12</v>
@@ -4769,7 +4769,7 @@
         <v>11</v>
       </c>
       <c r="E70" s="2">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F70" s="3" t="s">
         <v>12</v>
@@ -4795,7 +4795,7 @@
         <v>11</v>
       </c>
       <c r="E71" s="4">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>12</v>
@@ -4847,7 +4847,7 @@
         <v>11</v>
       </c>
       <c r="E73" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F73" s="3" t="s">
         <v>12</v>
@@ -4873,7 +4873,7 @@
         <v>11</v>
       </c>
       <c r="E74" s="2">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F74" s="3" t="s">
         <v>12</v>
@@ -4899,7 +4899,7 @@
         <v>11</v>
       </c>
       <c r="E75" s="4">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>12</v>
@@ -4925,7 +4925,7 @@
         <v>11</v>
       </c>
       <c r="E76" s="2">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F76" s="3" t="s">
         <v>12</v>
@@ -4951,7 +4951,7 @@
         <v>11</v>
       </c>
       <c r="E77" s="4">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>12</v>
@@ -4977,7 +4977,7 @@
         <v>11</v>
       </c>
       <c r="E78" s="2">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F78" s="3" t="s">
         <v>12</v>
@@ -5003,7 +5003,7 @@
         <v>11</v>
       </c>
       <c r="E79" s="4">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F79" s="3" t="s">
         <v>12</v>
@@ -5029,7 +5029,7 @@
         <v>11</v>
       </c>
       <c r="E80" s="2">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F80" s="3" t="s">
         <v>12</v>
@@ -5055,7 +5055,7 @@
         <v>11</v>
       </c>
       <c r="E81" s="4">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F81" s="3" t="s">
         <v>12</v>
@@ -5081,7 +5081,7 @@
         <v>11</v>
       </c>
       <c r="E82" s="2">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F82" s="3" t="s">
         <v>12</v>
@@ -5107,7 +5107,7 @@
         <v>11</v>
       </c>
       <c r="E83" s="4">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F83" s="3" t="s">
         <v>12</v>
@@ -5133,7 +5133,7 @@
         <v>11</v>
       </c>
       <c r="E84" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>12</v>
@@ -5159,7 +5159,7 @@
         <v>11</v>
       </c>
       <c r="E85" s="4">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>12</v>
@@ -5185,7 +5185,7 @@
         <v>11</v>
       </c>
       <c r="E86" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>12</v>
@@ -5211,7 +5211,7 @@
         <v>11</v>
       </c>
       <c r="E87" s="4">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>12</v>
@@ -5263,7 +5263,7 @@
         <v>11</v>
       </c>
       <c r="E89" s="4">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F89" s="3" t="s">
         <v>12</v>
@@ -5289,7 +5289,7 @@
         <v>11</v>
       </c>
       <c r="E90" s="2">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>12</v>
@@ -5315,7 +5315,7 @@
         <v>11</v>
       </c>
       <c r="E91" s="4">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F91" s="3" t="s">
         <v>12</v>
@@ -5341,7 +5341,7 @@
         <v>11</v>
       </c>
       <c r="E92" s="2">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F92" s="3" t="s">
         <v>12</v>
@@ -5367,7 +5367,7 @@
         <v>11</v>
       </c>
       <c r="E93" s="4">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F93" s="3" t="s">
         <v>12</v>
@@ -5393,7 +5393,7 @@
         <v>11</v>
       </c>
       <c r="E94" s="2">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F94" s="3" t="s">
         <v>12</v>
@@ -5419,7 +5419,7 @@
         <v>11</v>
       </c>
       <c r="E95" s="4">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F95" s="3" t="s">
         <v>12</v>
@@ -5445,7 +5445,7 @@
         <v>11</v>
       </c>
       <c r="E96" s="2">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F96" s="3" t="s">
         <v>12</v>
@@ -5497,7 +5497,7 @@
         <v>11</v>
       </c>
       <c r="E98" s="2">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>12</v>
@@ -5523,7 +5523,7 @@
         <v>11</v>
       </c>
       <c r="E99" s="4">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>12</v>
@@ -5549,7 +5549,7 @@
         <v>11</v>
       </c>
       <c r="E100" s="2">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>12</v>
@@ -5575,7 +5575,7 @@
         <v>11</v>
       </c>
       <c r="E101" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>12</v>
@@ -5601,7 +5601,7 @@
         <v>11</v>
       </c>
       <c r="E102" s="2">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>12</v>
@@ -5627,7 +5627,7 @@
         <v>11</v>
       </c>
       <c r="E103" s="4">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F103" s="3" t="s">
         <v>12</v>
@@ -5653,7 +5653,7 @@
         <v>11</v>
       </c>
       <c r="E104" s="2">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>12</v>
@@ -5679,7 +5679,7 @@
         <v>11</v>
       </c>
       <c r="E105" s="4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F105" s="3" t="s">
         <v>12</v>
@@ -5705,7 +5705,7 @@
         <v>11</v>
       </c>
       <c r="E106" s="2">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F106" s="3" t="s">
         <v>12</v>
@@ -5731,7 +5731,7 @@
         <v>11</v>
       </c>
       <c r="E107" s="4">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F107" s="3" t="s">
         <v>12</v>
@@ -5757,7 +5757,7 @@
         <v>11</v>
       </c>
       <c r="E108" s="2">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F108" s="3" t="s">
         <v>12</v>
@@ -5783,7 +5783,7 @@
         <v>11</v>
       </c>
       <c r="E109" s="4">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F109" s="3" t="s">
         <v>12</v>
@@ -5809,7 +5809,7 @@
         <v>11</v>
       </c>
       <c r="E110" s="2">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F110" s="3" t="s">
         <v>12</v>
@@ -5835,7 +5835,7 @@
         <v>11</v>
       </c>
       <c r="E111" s="4">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F111" s="3" t="s">
         <v>12</v>
@@ -5861,7 +5861,7 @@
         <v>11</v>
       </c>
       <c r="E112" s="2">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F112" s="3" t="s">
         <v>12</v>
@@ -5887,7 +5887,7 @@
         <v>11</v>
       </c>
       <c r="E113" s="4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F113" s="3" t="s">
         <v>12</v>
@@ -5913,7 +5913,7 @@
         <v>11</v>
       </c>
       <c r="E114" s="2">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F114" s="3" t="s">
         <v>12</v>
@@ -5939,7 +5939,7 @@
         <v>11</v>
       </c>
       <c r="E115" s="4">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>12</v>
@@ -5965,7 +5965,7 @@
         <v>11</v>
       </c>
       <c r="E116" s="2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F116" s="3" t="s">
         <v>12</v>
@@ -5991,7 +5991,7 @@
         <v>11</v>
       </c>
       <c r="E117" s="4">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>12</v>
@@ -6017,7 +6017,7 @@
         <v>11</v>
       </c>
       <c r="E118" s="2">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F118" s="3" t="s">
         <v>12</v>
@@ -6043,7 +6043,7 @@
         <v>11</v>
       </c>
       <c r="E119" s="4">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F119" s="3" t="s">
         <v>12</v>
@@ -6069,7 +6069,7 @@
         <v>11</v>
       </c>
       <c r="E120" s="2">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F120" s="3" t="s">
         <v>12</v>
@@ -6095,7 +6095,7 @@
         <v>11</v>
       </c>
       <c r="E121" s="4">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F121" s="3" t="s">
         <v>12</v>
@@ -6121,7 +6121,7 @@
         <v>11</v>
       </c>
       <c r="E122" s="2">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F122" s="3" t="s">
         <v>12</v>
@@ -6147,7 +6147,7 @@
         <v>11</v>
       </c>
       <c r="E123" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F123" s="3" t="s">
         <v>12</v>
@@ -6173,7 +6173,7 @@
         <v>11</v>
       </c>
       <c r="E124" s="2">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F124" s="3" t="s">
         <v>12</v>
@@ -6199,7 +6199,7 @@
         <v>11</v>
       </c>
       <c r="E125" s="4">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F125" s="3" t="s">
         <v>12</v>
@@ -6225,7 +6225,7 @@
         <v>11</v>
       </c>
       <c r="E126" s="2">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="F126" s="3" t="s">
         <v>12</v>
@@ -6251,7 +6251,7 @@
         <v>11</v>
       </c>
       <c r="E127" s="4">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F127" s="3" t="s">
         <v>12</v>
@@ -6277,7 +6277,7 @@
         <v>11</v>
       </c>
       <c r="E128" s="2">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F128" s="3" t="s">
         <v>12</v>
@@ -6303,7 +6303,7 @@
         <v>11</v>
       </c>
       <c r="E129" s="4">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F129" s="3" t="s">
         <v>12</v>
@@ -6329,7 +6329,7 @@
         <v>11</v>
       </c>
       <c r="E130" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>12</v>
@@ -6355,7 +6355,7 @@
         <v>11</v>
       </c>
       <c r="E131" s="4">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F131" s="3" t="s">
         <v>12</v>
@@ -6381,7 +6381,7 @@
         <v>11</v>
       </c>
       <c r="E132" s="2">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F132" s="3" t="s">
         <v>12</v>
@@ -6407,7 +6407,7 @@
         <v>11</v>
       </c>
       <c r="E133" s="4">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F133" s="3" t="s">
         <v>12</v>
@@ -6433,7 +6433,7 @@
         <v>11</v>
       </c>
       <c r="E134" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F134" s="3" t="s">
         <v>12</v>
@@ -6459,7 +6459,7 @@
         <v>11</v>
       </c>
       <c r="E135" s="4">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F135" s="3" t="s">
         <v>12</v>
@@ -6485,7 +6485,7 @@
         <v>11</v>
       </c>
       <c r="E136" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F136" s="3" t="s">
         <v>12</v>
@@ -6511,7 +6511,7 @@
         <v>11</v>
       </c>
       <c r="E137" s="4">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F137" s="3" t="s">
         <v>12</v>
@@ -6537,7 +6537,7 @@
         <v>11</v>
       </c>
       <c r="E138" s="2">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="F138" s="3" t="s">
         <v>12</v>
@@ -6563,7 +6563,7 @@
         <v>11</v>
       </c>
       <c r="E139" s="4">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="F139" s="3" t="s">
         <v>12</v>
@@ -6589,7 +6589,7 @@
         <v>11</v>
       </c>
       <c r="E140" s="2">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F140" s="3" t="s">
         <v>12</v>
@@ -6615,7 +6615,7 @@
         <v>11</v>
       </c>
       <c r="E141" s="4">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F141" s="3" t="s">
         <v>12</v>
@@ -6641,7 +6641,7 @@
         <v>11</v>
       </c>
       <c r="E142" s="2">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F142" s="3" t="s">
         <v>12</v>
@@ -6667,7 +6667,7 @@
         <v>11</v>
       </c>
       <c r="E143" s="4">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F143" s="3" t="s">
         <v>12</v>
@@ -6693,7 +6693,7 @@
         <v>11</v>
       </c>
       <c r="E144" s="2">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>12</v>
@@ -6719,7 +6719,7 @@
         <v>11</v>
       </c>
       <c r="E145" s="4">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F145" s="3" t="s">
         <v>12</v>
@@ -6745,7 +6745,7 @@
         <v>11</v>
       </c>
       <c r="E146" s="2">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F146" s="3" t="s">
         <v>12</v>
@@ -6771,7 +6771,7 @@
         <v>11</v>
       </c>
       <c r="E147" s="4">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F147" s="3" t="s">
         <v>12</v>
@@ -6797,7 +6797,7 @@
         <v>11</v>
       </c>
       <c r="E148" s="2">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>12</v>
@@ -6823,7 +6823,7 @@
         <v>11</v>
       </c>
       <c r="E149" s="4">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F149" s="3" t="s">
         <v>12</v>
@@ -6849,7 +6849,7 @@
         <v>11</v>
       </c>
       <c r="E150" s="2">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F150" s="3" t="s">
         <v>12</v>
@@ -6875,7 +6875,7 @@
         <v>11</v>
       </c>
       <c r="E151" s="4">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F151" s="3" t="s">
         <v>12</v>
@@ -6901,7 +6901,7 @@
         <v>11</v>
       </c>
       <c r="E152" s="2">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F152" s="3" t="s">
         <v>12</v>
@@ -6953,7 +6953,7 @@
         <v>11</v>
       </c>
       <c r="E154" s="2">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="F154" s="3" t="s">
         <v>12</v>
@@ -6979,7 +6979,7 @@
         <v>11</v>
       </c>
       <c r="E155" s="4">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F155" s="3" t="s">
         <v>12</v>
@@ -7031,7 +7031,7 @@
         <v>11</v>
       </c>
       <c r="E157" s="4">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F157" s="3" t="s">
         <v>12</v>
@@ -7057,7 +7057,7 @@
         <v>11</v>
       </c>
       <c r="E158" s="2">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F158" s="3" t="s">
         <v>12</v>
@@ -7083,7 +7083,7 @@
         <v>11</v>
       </c>
       <c r="E159" s="4">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F159" s="3" t="s">
         <v>12</v>
@@ -7109,7 +7109,7 @@
         <v>11</v>
       </c>
       <c r="E160" s="2">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F160" s="3" t="s">
         <v>12</v>
@@ -7135,7 +7135,7 @@
         <v>11</v>
       </c>
       <c r="E161" s="4">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F161" s="3" t="s">
         <v>12</v>
@@ -7161,7 +7161,7 @@
         <v>11</v>
       </c>
       <c r="E162" s="2">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F162" s="3" t="s">
         <v>12</v>
@@ -7187,7 +7187,7 @@
         <v>11</v>
       </c>
       <c r="E163" s="4">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F163" s="3" t="s">
         <v>12</v>
@@ -7213,7 +7213,7 @@
         <v>11</v>
       </c>
       <c r="E164" s="2">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F164" s="3" t="s">
         <v>12</v>
@@ -7239,7 +7239,7 @@
         <v>11</v>
       </c>
       <c r="E165" s="4">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F165" s="3" t="s">
         <v>12</v>
@@ -7265,7 +7265,7 @@
         <v>11</v>
       </c>
       <c r="E166" s="2">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F166" s="3" t="s">
         <v>12</v>
@@ -7291,7 +7291,7 @@
         <v>11</v>
       </c>
       <c r="E167" s="4">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F167" s="3" t="s">
         <v>12</v>
@@ -7317,7 +7317,7 @@
         <v>11</v>
       </c>
       <c r="E168" s="2">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F168" s="3" t="s">
         <v>12</v>
@@ -7343,7 +7343,7 @@
         <v>11</v>
       </c>
       <c r="E169" s="4">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F169" s="3" t="s">
         <v>12</v>
@@ -7369,7 +7369,7 @@
         <v>11</v>
       </c>
       <c r="E170" s="2">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F170" s="3" t="s">
         <v>12</v>
@@ -7395,7 +7395,7 @@
         <v>11</v>
       </c>
       <c r="E171" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F171" s="3" t="s">
         <v>12</v>
@@ -7447,7 +7447,7 @@
         <v>11</v>
       </c>
       <c r="E173" s="4">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F173" s="3" t="s">
         <v>12</v>
@@ -7473,7 +7473,7 @@
         <v>11</v>
       </c>
       <c r="E174" s="2">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F174" s="3" t="s">
         <v>12</v>
@@ -7525,7 +7525,7 @@
         <v>11</v>
       </c>
       <c r="E176" s="2">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F176" s="3" t="s">
         <v>12</v>
@@ -7551,7 +7551,7 @@
         <v>11</v>
       </c>
       <c r="E177" s="4">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F177" s="3" t="s">
         <v>12</v>
@@ -7577,7 +7577,7 @@
         <v>11</v>
       </c>
       <c r="E178" s="2">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F178" s="3" t="s">
         <v>12</v>
@@ -7629,7 +7629,7 @@
         <v>11</v>
       </c>
       <c r="E180" s="2">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F180" s="3" t="s">
         <v>12</v>
@@ -7655,7 +7655,7 @@
         <v>11</v>
       </c>
       <c r="E181" s="4">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F181" s="3" t="s">
         <v>12</v>
@@ -7681,7 +7681,7 @@
         <v>11</v>
       </c>
       <c r="E182" s="2">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F182" s="3" t="s">
         <v>12</v>
@@ -7707,7 +7707,7 @@
         <v>11</v>
       </c>
       <c r="E183" s="4">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F183" s="3" t="s">
         <v>12</v>
@@ -7733,7 +7733,7 @@
         <v>11</v>
       </c>
       <c r="E184" s="2">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F184" s="3" t="s">
         <v>12</v>
@@ -7785,7 +7785,7 @@
         <v>11</v>
       </c>
       <c r="E186" s="2">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F186" s="3" t="s">
         <v>12</v>
@@ -7811,7 +7811,7 @@
         <v>11</v>
       </c>
       <c r="E187" s="4">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F187" s="3" t="s">
         <v>12</v>
@@ -7837,7 +7837,7 @@
         <v>11</v>
       </c>
       <c r="E188" s="2">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F188" s="3" t="s">
         <v>12</v>
@@ -7863,7 +7863,7 @@
         <v>11</v>
       </c>
       <c r="E189" s="4">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F189" s="3" t="s">
         <v>12</v>
@@ -7889,7 +7889,7 @@
         <v>11</v>
       </c>
       <c r="E190" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F190" s="3" t="s">
         <v>12</v>
@@ -7915,7 +7915,7 @@
         <v>11</v>
       </c>
       <c r="E191" s="4">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F191" s="3" t="s">
         <v>12</v>
@@ -7941,7 +7941,7 @@
         <v>11</v>
       </c>
       <c r="E192" s="2">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F192" s="3" t="s">
         <v>12</v>
@@ -7967,7 +7967,7 @@
         <v>11</v>
       </c>
       <c r="E193" s="4">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F193" s="3" t="s">
         <v>12</v>
@@ -7993,7 +7993,7 @@
         <v>11</v>
       </c>
       <c r="E194" s="2">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F194" s="3" t="s">
         <v>12</v>
@@ -8019,7 +8019,7 @@
         <v>11</v>
       </c>
       <c r="E195" s="4">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F195" s="3" t="s">
         <v>12</v>
@@ -8045,7 +8045,7 @@
         <v>11</v>
       </c>
       <c r="E196" s="2">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F196" s="3" t="s">
         <v>12</v>
@@ -8071,7 +8071,7 @@
         <v>11</v>
       </c>
       <c r="E197" s="4">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F197" s="3" t="s">
         <v>12</v>
@@ -8097,7 +8097,7 @@
         <v>11</v>
       </c>
       <c r="E198" s="2">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F198" s="3" t="s">
         <v>12</v>
@@ -8123,7 +8123,7 @@
         <v>11</v>
       </c>
       <c r="E199" s="4">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="F199" s="3" t="s">
         <v>12</v>
@@ -8149,7 +8149,7 @@
         <v>11</v>
       </c>
       <c r="E200" s="2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F200" s="3" t="s">
         <v>12</v>
@@ -8175,7 +8175,7 @@
         <v>11</v>
       </c>
       <c r="E201" s="4">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F201" s="3" t="s">
         <v>12</v>
@@ -8201,7 +8201,7 @@
         <v>11</v>
       </c>
       <c r="E202" s="2">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F202" s="3" t="s">
         <v>12</v>
@@ -8227,7 +8227,7 @@
         <v>11</v>
       </c>
       <c r="E203" s="4">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F203" s="3" t="s">
         <v>12</v>
@@ -8253,7 +8253,7 @@
         <v>11</v>
       </c>
       <c r="E204" s="2">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F204" s="3" t="s">
         <v>12</v>
@@ -8279,7 +8279,7 @@
         <v>11</v>
       </c>
       <c r="E205" s="4">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F205" s="3" t="s">
         <v>12</v>
@@ -8305,7 +8305,7 @@
         <v>11</v>
       </c>
       <c r="E206" s="2">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F206" s="3" t="s">
         <v>12</v>
@@ -8331,7 +8331,7 @@
         <v>11</v>
       </c>
       <c r="E207" s="4">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F207" s="3" t="s">
         <v>12</v>
@@ -8357,7 +8357,7 @@
         <v>11</v>
       </c>
       <c r="E208" s="2">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F208" s="3" t="s">
         <v>12</v>
@@ -8383,7 +8383,7 @@
         <v>11</v>
       </c>
       <c r="E209" s="4">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F209" s="3" t="s">
         <v>12</v>
@@ -8409,7 +8409,7 @@
         <v>11</v>
       </c>
       <c r="E210" s="2">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F210" s="3" t="s">
         <v>12</v>
@@ -8435,7 +8435,7 @@
         <v>11</v>
       </c>
       <c r="E211" s="4">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F211" s="3" t="s">
         <v>12</v>
@@ -8461,7 +8461,7 @@
         <v>11</v>
       </c>
       <c r="E212" s="2">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F212" s="3" t="s">
         <v>12</v>
@@ -8487,7 +8487,7 @@
         <v>11</v>
       </c>
       <c r="E213" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F213" s="3" t="s">
         <v>12</v>
@@ -8513,7 +8513,7 @@
         <v>11</v>
       </c>
       <c r="E214" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F214" s="3" t="s">
         <v>12</v>
@@ -8539,7 +8539,7 @@
         <v>11</v>
       </c>
       <c r="E215" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F215" s="3" t="s">
         <v>12</v>
@@ -8565,7 +8565,7 @@
         <v>11</v>
       </c>
       <c r="E216" s="2">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F216" s="3" t="s">
         <v>12</v>
@@ -8591,7 +8591,7 @@
         <v>11</v>
       </c>
       <c r="E217" s="4">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="F217" s="3" t="s">
         <v>12</v>
@@ -8617,7 +8617,7 @@
         <v>11</v>
       </c>
       <c r="E218" s="2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F218" s="3" t="s">
         <v>12</v>
@@ -8669,7 +8669,7 @@
         <v>11</v>
       </c>
       <c r="E220" s="2">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F220" s="3" t="s">
         <v>12</v>
@@ -8695,7 +8695,7 @@
         <v>11</v>
       </c>
       <c r="E221" s="4">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F221" s="3" t="s">
         <v>12</v>
@@ -8721,7 +8721,7 @@
         <v>11</v>
       </c>
       <c r="E222" s="2">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F222" s="3" t="s">
         <v>12</v>
@@ -8747,7 +8747,7 @@
         <v>11</v>
       </c>
       <c r="E223" s="4">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F223" s="3" t="s">
         <v>12</v>
@@ -8773,7 +8773,7 @@
         <v>11</v>
       </c>
       <c r="E224" s="2">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F224" s="3" t="s">
         <v>12</v>
@@ -8799,7 +8799,7 @@
         <v>11</v>
       </c>
       <c r="E225" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F225" s="3" t="s">
         <v>12</v>
@@ -8825,7 +8825,7 @@
         <v>11</v>
       </c>
       <c r="E226" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F226" s="3" t="s">
         <v>12</v>
@@ -8851,7 +8851,7 @@
         <v>11</v>
       </c>
       <c r="E227" s="4">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F227" s="3" t="s">
         <v>12</v>
@@ -8903,7 +8903,7 @@
         <v>11</v>
       </c>
       <c r="E229" s="4">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="F229" s="3" t="s">
         <v>12</v>
@@ -8929,7 +8929,7 @@
         <v>11</v>
       </c>
       <c r="E230" s="2">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="F230" s="3" t="s">
         <v>12</v>
@@ -8955,7 +8955,7 @@
         <v>11</v>
       </c>
       <c r="E231" s="4">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F231" s="3" t="s">
         <v>12</v>
@@ -8981,7 +8981,7 @@
         <v>11</v>
       </c>
       <c r="E232" s="2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F232" s="3" t="s">
         <v>12</v>
@@ -9007,7 +9007,7 @@
         <v>11</v>
       </c>
       <c r="E233" s="4">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F233" s="3" t="s">
         <v>12</v>
@@ -9033,7 +9033,7 @@
         <v>11</v>
       </c>
       <c r="E234" s="2">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F234" s="3" t="s">
         <v>12</v>
@@ -9059,7 +9059,7 @@
         <v>11</v>
       </c>
       <c r="E235" s="4">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="F235" s="3" t="s">
         <v>12</v>
@@ -9085,7 +9085,7 @@
         <v>11</v>
       </c>
       <c r="E236" s="2">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F236" s="3" t="s">
         <v>12</v>
@@ -9111,7 +9111,7 @@
         <v>11</v>
       </c>
       <c r="E237" s="4">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F237" s="3" t="s">
         <v>12</v>
@@ -9137,7 +9137,7 @@
         <v>11</v>
       </c>
       <c r="E238" s="2">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F238" s="3" t="s">
         <v>12</v>
@@ -9163,7 +9163,7 @@
         <v>11</v>
       </c>
       <c r="E239" s="4">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F239" s="3" t="s">
         <v>12</v>
@@ -9189,7 +9189,7 @@
         <v>11</v>
       </c>
       <c r="E240" s="2">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F240" s="3" t="s">
         <v>12</v>
@@ -9215,7 +9215,7 @@
         <v>11</v>
       </c>
       <c r="E241" s="4">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F241" s="3" t="s">
         <v>12</v>
@@ -9241,7 +9241,7 @@
         <v>11</v>
       </c>
       <c r="E242" s="2">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F242" s="3" t="s">
         <v>12</v>
@@ -9267,7 +9267,7 @@
         <v>11</v>
       </c>
       <c r="E243" s="4">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F243" s="3" t="s">
         <v>12</v>
@@ -9293,7 +9293,7 @@
         <v>11</v>
       </c>
       <c r="E244" s="2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F244" s="3" t="s">
         <v>12</v>
@@ -9319,7 +9319,7 @@
         <v>11</v>
       </c>
       <c r="E245" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F245" s="3" t="s">
         <v>12</v>
@@ -9345,7 +9345,7 @@
         <v>11</v>
       </c>
       <c r="E246" s="2">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F246" s="3" t="s">
         <v>12</v>
@@ -9371,7 +9371,7 @@
         <v>11</v>
       </c>
       <c r="E247" s="4">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F247" s="3" t="s">
         <v>12</v>
@@ -9397,7 +9397,7 @@
         <v>11</v>
       </c>
       <c r="E248" s="2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F248" s="3" t="s">
         <v>12</v>
@@ -9423,7 +9423,7 @@
         <v>11</v>
       </c>
       <c r="E249" s="4">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F249" s="3" t="s">
         <v>12</v>
@@ -9449,7 +9449,7 @@
         <v>11</v>
       </c>
       <c r="E250" s="2">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F250" s="3" t="s">
         <v>12</v>
@@ -9475,7 +9475,7 @@
         <v>11</v>
       </c>
       <c r="E251" s="4">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F251" s="3" t="s">
         <v>12</v>
@@ -9501,7 +9501,7 @@
         <v>11</v>
       </c>
       <c r="E252" s="2">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F252" s="3" t="s">
         <v>12</v>
@@ -9527,7 +9527,7 @@
         <v>11</v>
       </c>
       <c r="E253" s="4">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F253" s="3" t="s">
         <v>12</v>
@@ -9553,7 +9553,7 @@
         <v>11</v>
       </c>
       <c r="E254" s="2">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F254" s="3" t="s">
         <v>12</v>
@@ -9579,7 +9579,7 @@
         <v>11</v>
       </c>
       <c r="E255" s="4">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>12</v>
@@ -9605,7 +9605,7 @@
         <v>11</v>
       </c>
       <c r="E256" s="2">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F256" s="3" t="s">
         <v>12</v>
@@ -9631,7 +9631,7 @@
         <v>11</v>
       </c>
       <c r="E257" s="4">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F257" s="3" t="s">
         <v>12</v>
@@ -9657,7 +9657,7 @@
         <v>11</v>
       </c>
       <c r="E258" s="2">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F258" s="3" t="s">
         <v>12</v>
@@ -9683,7 +9683,7 @@
         <v>11</v>
       </c>
       <c r="E259" s="4">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F259" s="3" t="s">
         <v>12</v>
@@ -9709,7 +9709,7 @@
         <v>11</v>
       </c>
       <c r="E260" s="2">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F260" s="3" t="s">
         <v>12</v>
@@ -9735,7 +9735,7 @@
         <v>11</v>
       </c>
       <c r="E261" s="4">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F261" s="3" t="s">
         <v>12</v>
@@ -9761,7 +9761,7 @@
         <v>11</v>
       </c>
       <c r="E262" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F262" s="3" t="s">
         <v>12</v>
@@ -9787,7 +9787,7 @@
         <v>11</v>
       </c>
       <c r="E263" s="4">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F263" s="3" t="s">
         <v>12</v>
@@ -9813,7 +9813,7 @@
         <v>11</v>
       </c>
       <c r="E264" s="2">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F264" s="3" t="s">
         <v>12</v>
@@ -9839,7 +9839,7 @@
         <v>11</v>
       </c>
       <c r="E265" s="4">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F265" s="3" t="s">
         <v>12</v>
@@ -9891,7 +9891,7 @@
         <v>11</v>
       </c>
       <c r="E267" s="4">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F267" s="3" t="s">
         <v>12</v>
@@ -9917,7 +9917,7 @@
         <v>11</v>
       </c>
       <c r="E268" s="2">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F268" s="3" t="s">
         <v>12</v>
@@ -9943,7 +9943,7 @@
         <v>11</v>
       </c>
       <c r="E269" s="4">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F269" s="3" t="s">
         <v>12</v>
@@ -9969,7 +9969,7 @@
         <v>11</v>
       </c>
       <c r="E270" s="2">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F270" s="3" t="s">
         <v>12</v>
@@ -9995,7 +9995,7 @@
         <v>11</v>
       </c>
       <c r="E271" s="4">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F271" s="3" t="s">
         <v>12</v>
@@ -10021,7 +10021,7 @@
         <v>11</v>
       </c>
       <c r="E272" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F272" s="3" t="s">
         <v>12</v>
@@ -10047,7 +10047,7 @@
         <v>11</v>
       </c>
       <c r="E273" s="4">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F273" s="3" t="s">
         <v>12</v>
@@ -10099,7 +10099,7 @@
         <v>11</v>
       </c>
       <c r="E275" s="4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F275" s="3" t="s">
         <v>12</v>
@@ -10125,7 +10125,7 @@
         <v>11</v>
       </c>
       <c r="E276" s="2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F276" s="3" t="s">
         <v>12</v>
@@ -10151,7 +10151,7 @@
         <v>11</v>
       </c>
       <c r="E277" s="4">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F277" s="3" t="s">
         <v>12</v>
@@ -10177,7 +10177,7 @@
         <v>11</v>
       </c>
       <c r="E278" s="2">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F278" s="3" t="s">
         <v>12</v>
@@ -10203,7 +10203,7 @@
         <v>11</v>
       </c>
       <c r="E279" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F279" s="3" t="s">
         <v>12</v>
@@ -10229,7 +10229,7 @@
         <v>11</v>
       </c>
       <c r="E280" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F280" s="3" t="s">
         <v>12</v>
@@ -10255,7 +10255,7 @@
         <v>11</v>
       </c>
       <c r="E281" s="4">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F281" s="3" t="s">
         <v>12</v>
@@ -10281,7 +10281,7 @@
         <v>11</v>
       </c>
       <c r="E282" s="2">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F282" s="3" t="s">
         <v>12</v>
@@ -10307,7 +10307,7 @@
         <v>11</v>
       </c>
       <c r="E283" s="4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F283" s="3" t="s">
         <v>12</v>
@@ -10333,7 +10333,7 @@
         <v>11</v>
       </c>
       <c r="E284" s="2">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F284" s="3" t="s">
         <v>12</v>
@@ -10359,7 +10359,7 @@
         <v>11</v>
       </c>
       <c r="E285" s="4">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F285" s="3" t="s">
         <v>12</v>
@@ -10385,7 +10385,7 @@
         <v>11</v>
       </c>
       <c r="E286" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F286" s="3" t="s">
         <v>12</v>
@@ -10411,7 +10411,7 @@
         <v>11</v>
       </c>
       <c r="E287" s="4">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F287" s="3" t="s">
         <v>12</v>
@@ -10437,7 +10437,7 @@
         <v>11</v>
       </c>
       <c r="E288" s="2">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="F288" s="3" t="s">
         <v>12</v>
@@ -10489,7 +10489,7 @@
         <v>11</v>
       </c>
       <c r="E290" s="2">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F290" s="3" t="s">
         <v>12</v>
@@ -10515,7 +10515,7 @@
         <v>11</v>
       </c>
       <c r="E291" s="4">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="F291" s="3" t="s">
         <v>12</v>
@@ -10541,7 +10541,7 @@
         <v>11</v>
       </c>
       <c r="E292" s="2">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F292" s="3" t="s">
         <v>12</v>
@@ -10567,7 +10567,7 @@
         <v>11</v>
       </c>
       <c r="E293" s="4">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F293" s="3" t="s">
         <v>12</v>
@@ -10593,7 +10593,7 @@
         <v>11</v>
       </c>
       <c r="E294" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F294" s="3" t="s">
         <v>12</v>
@@ -10619,7 +10619,7 @@
         <v>11</v>
       </c>
       <c r="E295" s="4">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F295" s="3" t="s">
         <v>12</v>
@@ -10645,7 +10645,7 @@
         <v>11</v>
       </c>
       <c r="E296" s="2">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F296" s="3" t="s">
         <v>12</v>
@@ -10671,7 +10671,7 @@
         <v>11</v>
       </c>
       <c r="E297" s="4">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="F297" s="3" t="s">
         <v>12</v>
@@ -10697,7 +10697,7 @@
         <v>11</v>
       </c>
       <c r="E298" s="2">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F298" s="3" t="s">
         <v>12</v>
@@ -10723,7 +10723,7 @@
         <v>11</v>
       </c>
       <c r="E299" s="4">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F299" s="3" t="s">
         <v>12</v>
@@ -10749,7 +10749,7 @@
         <v>11</v>
       </c>
       <c r="E300" s="2">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F300" s="3" t="s">
         <v>12</v>
@@ -10775,7 +10775,7 @@
         <v>11</v>
       </c>
       <c r="E301" s="4">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F301" s="3" t="s">
         <v>12</v>
@@ -10801,7 +10801,7 @@
         <v>11</v>
       </c>
       <c r="E302" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F302" s="3" t="s">
         <v>12</v>
@@ -10827,7 +10827,7 @@
         <v>11</v>
       </c>
       <c r="E303" s="4">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F303" s="3" t="s">
         <v>12</v>
@@ -10853,7 +10853,7 @@
         <v>11</v>
       </c>
       <c r="E304" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F304" s="3" t="s">
         <v>12</v>
@@ -10879,7 +10879,7 @@
         <v>11</v>
       </c>
       <c r="E305" s="4">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F305" s="3" t="s">
         <v>12</v>
@@ -10905,7 +10905,7 @@
         <v>11</v>
       </c>
       <c r="E306" s="2">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F306" s="3" t="s">
         <v>12</v>
@@ -10931,7 +10931,7 @@
         <v>11</v>
       </c>
       <c r="E307" s="4">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F307" s="3" t="s">
         <v>12</v>
@@ -10957,7 +10957,7 @@
         <v>11</v>
       </c>
       <c r="E308" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F308" s="3" t="s">
         <v>12</v>
@@ -10983,7 +10983,7 @@
         <v>11</v>
       </c>
       <c r="E309" s="4">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F309" s="3" t="s">
         <v>12</v>
@@ -11009,7 +11009,7 @@
         <v>11</v>
       </c>
       <c r="E310" s="2">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F310" s="3" t="s">
         <v>12</v>
@@ -11035,7 +11035,7 @@
         <v>11</v>
       </c>
       <c r="E311" s="4">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F311" s="3" t="s">
         <v>12</v>
@@ -11061,7 +11061,7 @@
         <v>11</v>
       </c>
       <c r="E312" s="2">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F312" s="3" t="s">
         <v>12</v>
@@ -11087,7 +11087,7 @@
         <v>11</v>
       </c>
       <c r="E313" s="4">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F313" s="3" t="s">
         <v>12</v>
@@ -11113,7 +11113,7 @@
         <v>11</v>
       </c>
       <c r="E314" s="2">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F314" s="3" t="s">
         <v>12</v>
@@ -11139,7 +11139,7 @@
         <v>11</v>
       </c>
       <c r="E315" s="4">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F315" s="3" t="s">
         <v>12</v>
@@ -11165,7 +11165,7 @@
         <v>11</v>
       </c>
       <c r="E316" s="2">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="F316" s="3" t="s">
         <v>12</v>
@@ -11191,7 +11191,7 @@
         <v>11</v>
       </c>
       <c r="E317" s="4">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F317" s="3" t="s">
         <v>12</v>
@@ -11217,7 +11217,7 @@
         <v>11</v>
       </c>
       <c r="E318" s="2">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F318" s="3" t="s">
         <v>12</v>
@@ -11243,7 +11243,7 @@
         <v>11</v>
       </c>
       <c r="E319" s="4">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F319" s="3" t="s">
         <v>12</v>
@@ -11321,7 +11321,7 @@
         <v>11</v>
       </c>
       <c r="E322" s="2">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F322" s="3" t="s">
         <v>12</v>
@@ -11347,7 +11347,7 @@
         <v>11</v>
       </c>
       <c r="E323" s="4">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F323" s="3" t="s">
         <v>12</v>
@@ -11373,7 +11373,7 @@
         <v>11</v>
       </c>
       <c r="E324" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F324" s="3" t="s">
         <v>12</v>
@@ -11399,7 +11399,7 @@
         <v>11</v>
       </c>
       <c r="E325" s="4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F325" s="3" t="s">
         <v>12</v>
@@ -11425,7 +11425,7 @@
         <v>11</v>
       </c>
       <c r="E326" s="2">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F326" s="3" t="s">
         <v>12</v>
@@ -11451,7 +11451,7 @@
         <v>11</v>
       </c>
       <c r="E327" s="4">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F327" s="3" t="s">
         <v>12</v>
@@ -11477,7 +11477,7 @@
         <v>11</v>
       </c>
       <c r="E328" s="2">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F328" s="3" t="s">
         <v>12</v>
@@ -11503,7 +11503,7 @@
         <v>11</v>
       </c>
       <c r="E329" s="4">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F329" s="3" t="s">
         <v>12</v>
@@ -11529,7 +11529,7 @@
         <v>11</v>
       </c>
       <c r="E330" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F330" s="3" t="s">
         <v>12</v>
@@ -11555,7 +11555,7 @@
         <v>11</v>
       </c>
       <c r="E331" s="4">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F331" s="3" t="s">
         <v>12</v>
@@ -11581,7 +11581,7 @@
         <v>11</v>
       </c>
       <c r="E332" s="2">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F332" s="3" t="s">
         <v>12</v>
@@ -11607,7 +11607,7 @@
         <v>11</v>
       </c>
       <c r="E333" s="4">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F333" s="3" t="s">
         <v>12</v>
@@ -11633,7 +11633,7 @@
         <v>11</v>
       </c>
       <c r="E334" s="2">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F334" s="3" t="s">
         <v>12</v>
@@ -11659,7 +11659,7 @@
         <v>11</v>
       </c>
       <c r="E335" s="4">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F335" s="3" t="s">
         <v>12</v>
@@ -11685,7 +11685,7 @@
         <v>11</v>
       </c>
       <c r="E336" s="2">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F336" s="3" t="s">
         <v>12</v>
@@ -11711,7 +11711,7 @@
         <v>11</v>
       </c>
       <c r="E337" s="4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F337" s="3" t="s">
         <v>12</v>
@@ -11737,7 +11737,7 @@
         <v>11</v>
       </c>
       <c r="E338" s="2">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F338" s="3" t="s">
         <v>12</v>
@@ -11763,7 +11763,7 @@
         <v>11</v>
       </c>
       <c r="E339" s="4">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F339" s="3" t="s">
         <v>12</v>
@@ -11789,7 +11789,7 @@
         <v>11</v>
       </c>
       <c r="E340" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F340" s="3" t="s">
         <v>12</v>
@@ -11815,7 +11815,7 @@
         <v>11</v>
       </c>
       <c r="E341" s="4">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F341" s="3" t="s">
         <v>12</v>
@@ -11841,7 +11841,7 @@
         <v>11</v>
       </c>
       <c r="E342" s="2">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F342" s="3" t="s">
         <v>12</v>
@@ -11867,7 +11867,7 @@
         <v>11</v>
       </c>
       <c r="E343" s="4">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F343" s="3" t="s">
         <v>12</v>
@@ -11893,7 +11893,7 @@
         <v>11</v>
       </c>
       <c r="E344" s="2">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F344" s="3" t="s">
         <v>12</v>
@@ -11919,7 +11919,7 @@
         <v>11</v>
       </c>
       <c r="E345" s="4">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F345" s="3" t="s">
         <v>12</v>
@@ -11945,7 +11945,7 @@
         <v>11</v>
       </c>
       <c r="E346" s="2">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F346" s="3" t="s">
         <v>12</v>
@@ -11971,7 +11971,7 @@
         <v>11</v>
       </c>
       <c r="E347" s="4">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F347" s="3" t="s">
         <v>12</v>
@@ -11997,7 +11997,7 @@
         <v>11</v>
       </c>
       <c r="E348" s="2">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F348" s="3" t="s">
         <v>12</v>
@@ -12023,7 +12023,7 @@
         <v>11</v>
       </c>
       <c r="E349" s="4">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F349" s="3" t="s">
         <v>12</v>
@@ -12049,7 +12049,7 @@
         <v>11</v>
       </c>
       <c r="E350" s="2">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F350" s="3" t="s">
         <v>12</v>
@@ -12075,7 +12075,7 @@
         <v>11</v>
       </c>
       <c r="E351" s="4">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F351" s="3" t="s">
         <v>12</v>
@@ -12101,7 +12101,7 @@
         <v>11</v>
       </c>
       <c r="E352" s="2">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F352" s="3" t="s">
         <v>12</v>
@@ -12127,7 +12127,7 @@
         <v>11</v>
       </c>
       <c r="E353" s="4">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F353" s="3" t="s">
         <v>12</v>
@@ -12153,7 +12153,7 @@
         <v>11</v>
       </c>
       <c r="E354" s="2">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F354" s="3" t="s">
         <v>12</v>
@@ -12205,7 +12205,7 @@
         <v>11</v>
       </c>
       <c r="E356" s="2">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F356" s="3" t="s">
         <v>12</v>
@@ -12231,7 +12231,7 @@
         <v>11</v>
       </c>
       <c r="E357" s="4">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F357" s="3" t="s">
         <v>12</v>
@@ -12283,7 +12283,7 @@
         <v>11</v>
       </c>
       <c r="E359" s="4">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F359" s="3" t="s">
         <v>12</v>
@@ -12309,7 +12309,7 @@
         <v>11</v>
       </c>
       <c r="E360" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F360" s="3" t="s">
         <v>12</v>
@@ -12335,7 +12335,7 @@
         <v>11</v>
       </c>
       <c r="E361" s="4">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F361" s="3" t="s">
         <v>12</v>
@@ -12361,7 +12361,7 @@
         <v>11</v>
       </c>
       <c r="E362" s="2">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F362" s="3" t="s">
         <v>12</v>
@@ -12387,7 +12387,7 @@
         <v>11</v>
       </c>
       <c r="E363" s="4">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F363" s="3" t="s">
         <v>12</v>
@@ -12413,7 +12413,7 @@
         <v>11</v>
       </c>
       <c r="E364" s="2">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F364" s="3" t="s">
         <v>12</v>
@@ -12439,7 +12439,7 @@
         <v>11</v>
       </c>
       <c r="E365" s="4">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F365" s="3" t="s">
         <v>12</v>
@@ -12465,7 +12465,7 @@
         <v>11</v>
       </c>
       <c r="E366" s="2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F366" s="3" t="s">
         <v>12</v>
@@ -12491,7 +12491,7 @@
         <v>11</v>
       </c>
       <c r="E367" s="4">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F367" s="3" t="s">
         <v>12</v>
@@ -12517,7 +12517,7 @@
         <v>11</v>
       </c>
       <c r="E368" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F368" s="3" t="s">
         <v>12</v>
@@ -12543,7 +12543,7 @@
         <v>11</v>
       </c>
       <c r="E369" s="4">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F369" s="3" t="s">
         <v>12</v>
@@ -12569,7 +12569,7 @@
         <v>11</v>
       </c>
       <c r="E370" s="2">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F370" s="3" t="s">
         <v>12</v>
@@ -12595,7 +12595,7 @@
         <v>11</v>
       </c>
       <c r="E371" s="4">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F371" s="3" t="s">
         <v>12</v>
@@ -12621,7 +12621,7 @@
         <v>11</v>
       </c>
       <c r="E372" s="2">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F372" s="3" t="s">
         <v>12</v>
@@ -12647,7 +12647,7 @@
         <v>11</v>
       </c>
       <c r="E373" s="4">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F373" s="3" t="s">
         <v>12</v>
@@ -12673,7 +12673,7 @@
         <v>11</v>
       </c>
       <c r="E374" s="2">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F374" s="3" t="s">
         <v>12</v>
@@ -12699,7 +12699,7 @@
         <v>11</v>
       </c>
       <c r="E375" s="4">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F375" s="3" t="s">
         <v>12</v>
@@ -12725,7 +12725,7 @@
         <v>11</v>
       </c>
       <c r="E376" s="2">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F376" s="3" t="s">
         <v>12</v>
@@ -12751,7 +12751,7 @@
         <v>11</v>
       </c>
       <c r="E377" s="4">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F377" s="3" t="s">
         <v>12</v>
@@ -12777,7 +12777,7 @@
         <v>11</v>
       </c>
       <c r="E378" s="2">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="F378" s="3" t="s">
         <v>12</v>
@@ -12803,7 +12803,7 @@
         <v>11</v>
       </c>
       <c r="E379" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F379" s="3" t="s">
         <v>12</v>
@@ -12829,7 +12829,7 @@
         <v>11</v>
       </c>
       <c r="E380" s="2">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F380" s="3" t="s">
         <v>12</v>
@@ -12855,7 +12855,7 @@
         <v>11</v>
       </c>
       <c r="E381" s="4">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F381" s="3" t="s">
         <v>12</v>
@@ -12881,7 +12881,7 @@
         <v>11</v>
       </c>
       <c r="E382" s="2">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F382" s="3" t="s">
         <v>12</v>
@@ -12907,7 +12907,7 @@
         <v>11</v>
       </c>
       <c r="E383" s="4">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F383" s="3" t="s">
         <v>12</v>
@@ -12933,7 +12933,7 @@
         <v>11</v>
       </c>
       <c r="E384" s="2">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F384" s="3" t="s">
         <v>12</v>
@@ -12959,7 +12959,7 @@
         <v>11</v>
       </c>
       <c r="E385" s="4">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F385" s="3" t="s">
         <v>12</v>
@@ -12985,7 +12985,7 @@
         <v>11</v>
       </c>
       <c r="E386" s="2">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F386" s="3" t="s">
         <v>12</v>
@@ -13011,7 +13011,7 @@
         <v>11</v>
       </c>
       <c r="E387" s="4">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F387" s="3" t="s">
         <v>12</v>
@@ -13037,7 +13037,7 @@
         <v>11</v>
       </c>
       <c r="E388" s="2">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F388" s="3" t="s">
         <v>12</v>
@@ -13063,7 +13063,7 @@
         <v>11</v>
       </c>
       <c r="E389" s="4">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F389" s="3" t="s">
         <v>12</v>
@@ -13089,7 +13089,7 @@
         <v>11</v>
       </c>
       <c r="E390" s="2">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F390" s="3" t="s">
         <v>12</v>
@@ -13115,7 +13115,7 @@
         <v>11</v>
       </c>
       <c r="E391" s="4">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F391" s="3" t="s">
         <v>12</v>
@@ -13141,7 +13141,7 @@
         <v>11</v>
       </c>
       <c r="E392" s="2">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F392" s="3" t="s">
         <v>12</v>
@@ -13167,7 +13167,7 @@
         <v>11</v>
       </c>
       <c r="E393" s="4">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F393" s="3" t="s">
         <v>12</v>
@@ -13193,7 +13193,7 @@
         <v>11</v>
       </c>
       <c r="E394" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F394" s="3" t="s">
         <v>12</v>
@@ -13219,7 +13219,7 @@
         <v>11</v>
       </c>
       <c r="E395" s="4">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F395" s="3" t="s">
         <v>12</v>
@@ -13245,7 +13245,7 @@
         <v>11</v>
       </c>
       <c r="E396" s="2">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F396" s="3" t="s">
         <v>12</v>
@@ -13271,7 +13271,7 @@
         <v>11</v>
       </c>
       <c r="E397" s="4">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F397" s="3" t="s">
         <v>12</v>
@@ -13297,7 +13297,7 @@
         <v>11</v>
       </c>
       <c r="E398" s="2">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F398" s="3" t="s">
         <v>12</v>
@@ -13323,7 +13323,7 @@
         <v>11</v>
       </c>
       <c r="E399" s="4">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F399" s="3" t="s">
         <v>12</v>
@@ -13349,7 +13349,7 @@
         <v>11</v>
       </c>
       <c r="E400" s="2">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F400" s="3" t="s">
         <v>12</v>
@@ -13375,7 +13375,7 @@
         <v>11</v>
       </c>
       <c r="E401" s="4">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F401" s="3" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ tarun2184/DEVLINK@5a49c57c251f6aff4cdec033f773aca0d05dd7d6 🚀
</commit_message>
<xml_diff>
--- a/reports/Mobile_Appium_E2E_Test_Report_400.xlsx
+++ b/reports/Mobile_Appium_E2E_Test_Report_400.xlsx
@@ -52,7 +52,7 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-08-10T08:42:32.516Z</t>
+    <t>2026-08-21T07:56:03.570Z</t>
   </si>
   <si>
     <t>Verified Android Activity lifecycle and Capacitor native plugin interface</t>
@@ -3001,7 +3001,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>12</v>
@@ -3027,7 +3027,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="4">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>12</v>
@@ -3053,7 +3053,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>12</v>
@@ -3105,7 +3105,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>12</v>
@@ -3131,7 +3131,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="4">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>12</v>
@@ -3157,7 +3157,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="2">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>12</v>
@@ -3183,7 +3183,7 @@
         <v>11</v>
       </c>
       <c r="E9" s="4">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>12</v>
@@ -3209,7 +3209,7 @@
         <v>11</v>
       </c>
       <c r="E10" s="2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>12</v>
@@ -3235,7 +3235,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="4">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>12</v>
@@ -3287,7 +3287,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="4">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>12</v>
@@ -3313,7 +3313,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="2">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>12</v>
@@ -3339,7 +3339,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="4">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>12</v>
@@ -3365,7 +3365,7 @@
         <v>11</v>
       </c>
       <c r="E16" s="2">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>12</v>
@@ -3391,7 +3391,7 @@
         <v>11</v>
       </c>
       <c r="E17" s="4">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>12</v>
@@ -3417,7 +3417,7 @@
         <v>11</v>
       </c>
       <c r="E18" s="2">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>12</v>
@@ -3443,7 +3443,7 @@
         <v>11</v>
       </c>
       <c r="E19" s="4">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>12</v>
@@ -3495,7 +3495,7 @@
         <v>11</v>
       </c>
       <c r="E21" s="4">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>12</v>
@@ -3521,7 +3521,7 @@
         <v>11</v>
       </c>
       <c r="E22" s="2">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>12</v>
@@ -3547,7 +3547,7 @@
         <v>11</v>
       </c>
       <c r="E23" s="4">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>12</v>
@@ -3573,7 +3573,7 @@
         <v>11</v>
       </c>
       <c r="E24" s="2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>12</v>
@@ -3599,7 +3599,7 @@
         <v>11</v>
       </c>
       <c r="E25" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>12</v>
@@ -3625,7 +3625,7 @@
         <v>11</v>
       </c>
       <c r="E26" s="2">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>12</v>
@@ -3703,7 +3703,7 @@
         <v>11</v>
       </c>
       <c r="E29" s="4">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>12</v>
@@ -3729,7 +3729,7 @@
         <v>11</v>
       </c>
       <c r="E30" s="2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>12</v>
@@ -3755,7 +3755,7 @@
         <v>11</v>
       </c>
       <c r="E31" s="4">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>12</v>
@@ -3781,7 +3781,7 @@
         <v>11</v>
       </c>
       <c r="E32" s="2">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>12</v>
@@ -3807,7 +3807,7 @@
         <v>11</v>
       </c>
       <c r="E33" s="4">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>12</v>
@@ -3833,7 +3833,7 @@
         <v>11</v>
       </c>
       <c r="E34" s="2">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>12</v>
@@ -3859,7 +3859,7 @@
         <v>11</v>
       </c>
       <c r="E35" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>12</v>
@@ -3885,7 +3885,7 @@
         <v>11</v>
       </c>
       <c r="E36" s="2">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>12</v>
@@ -3911,7 +3911,7 @@
         <v>11</v>
       </c>
       <c r="E37" s="4">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>12</v>
@@ -3937,7 +3937,7 @@
         <v>11</v>
       </c>
       <c r="E38" s="2">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>12</v>
@@ -3963,7 +3963,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="4">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>12</v>
@@ -4015,7 +4015,7 @@
         <v>11</v>
       </c>
       <c r="E41" s="4">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>12</v>
@@ -4041,7 +4041,7 @@
         <v>11</v>
       </c>
       <c r="E42" s="2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>12</v>
@@ -4067,7 +4067,7 @@
         <v>11</v>
       </c>
       <c r="E43" s="4">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>12</v>
@@ -4093,7 +4093,7 @@
         <v>11</v>
       </c>
       <c r="E44" s="2">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>12</v>
@@ -4119,7 +4119,7 @@
         <v>11</v>
       </c>
       <c r="E45" s="4">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>12</v>
@@ -4145,7 +4145,7 @@
         <v>11</v>
       </c>
       <c r="E46" s="2">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>12</v>
@@ -4171,7 +4171,7 @@
         <v>11</v>
       </c>
       <c r="E47" s="4">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>12</v>
@@ -4197,7 +4197,7 @@
         <v>11</v>
       </c>
       <c r="E48" s="2">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>12</v>
@@ -4249,7 +4249,7 @@
         <v>11</v>
       </c>
       <c r="E50" s="2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F50" s="3" t="s">
         <v>12</v>
@@ -4275,7 +4275,7 @@
         <v>11</v>
       </c>
       <c r="E51" s="4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>12</v>
@@ -4301,7 +4301,7 @@
         <v>11</v>
       </c>
       <c r="E52" s="2">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>12</v>
@@ -4327,7 +4327,7 @@
         <v>11</v>
       </c>
       <c r="E53" s="4">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>12</v>
@@ -4353,7 +4353,7 @@
         <v>11</v>
       </c>
       <c r="E54" s="2">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>12</v>
@@ -4379,7 +4379,7 @@
         <v>11</v>
       </c>
       <c r="E55" s="4">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F55" s="3" t="s">
         <v>12</v>
@@ -4405,7 +4405,7 @@
         <v>11</v>
       </c>
       <c r="E56" s="2">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>12</v>
@@ -4457,7 +4457,7 @@
         <v>11</v>
       </c>
       <c r="E58" s="2">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>12</v>
@@ -4483,7 +4483,7 @@
         <v>11</v>
       </c>
       <c r="E59" s="4">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>12</v>
@@ -4509,7 +4509,7 @@
         <v>11</v>
       </c>
       <c r="E60" s="2">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>12</v>
@@ -4535,7 +4535,7 @@
         <v>11</v>
       </c>
       <c r="E61" s="4">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>12</v>
@@ -4561,7 +4561,7 @@
         <v>11</v>
       </c>
       <c r="E62" s="2">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>12</v>
@@ -4587,7 +4587,7 @@
         <v>11</v>
       </c>
       <c r="E63" s="4">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>12</v>
@@ -4613,7 +4613,7 @@
         <v>11</v>
       </c>
       <c r="E64" s="2">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>12</v>
@@ -4639,7 +4639,7 @@
         <v>11</v>
       </c>
       <c r="E65" s="4">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>12</v>
@@ -4665,7 +4665,7 @@
         <v>11</v>
       </c>
       <c r="E66" s="2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>12</v>
@@ -4691,7 +4691,7 @@
         <v>11</v>
       </c>
       <c r="E67" s="4">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>12</v>
@@ -4743,7 +4743,7 @@
         <v>11</v>
       </c>
       <c r="E69" s="4">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>12</v>
@@ -4769,7 +4769,7 @@
         <v>11</v>
       </c>
       <c r="E70" s="2">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F70" s="3" t="s">
         <v>12</v>
@@ -4795,7 +4795,7 @@
         <v>11</v>
       </c>
       <c r="E71" s="4">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F71" s="3" t="s">
         <v>12</v>
@@ -4821,7 +4821,7 @@
         <v>11</v>
       </c>
       <c r="E72" s="2">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F72" s="3" t="s">
         <v>12</v>
@@ -4847,7 +4847,7 @@
         <v>11</v>
       </c>
       <c r="E73" s="4">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F73" s="3" t="s">
         <v>12</v>
@@ -4873,7 +4873,7 @@
         <v>11</v>
       </c>
       <c r="E74" s="2">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="F74" s="3" t="s">
         <v>12</v>
@@ -4899,7 +4899,7 @@
         <v>11</v>
       </c>
       <c r="E75" s="4">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F75" s="3" t="s">
         <v>12</v>
@@ -4925,7 +4925,7 @@
         <v>11</v>
       </c>
       <c r="E76" s="2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F76" s="3" t="s">
         <v>12</v>
@@ -4951,7 +4951,7 @@
         <v>11</v>
       </c>
       <c r="E77" s="4">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>12</v>
@@ -4977,7 +4977,7 @@
         <v>11</v>
       </c>
       <c r="E78" s="2">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F78" s="3" t="s">
         <v>12</v>
@@ -5003,7 +5003,7 @@
         <v>11</v>
       </c>
       <c r="E79" s="4">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F79" s="3" t="s">
         <v>12</v>
@@ -5029,7 +5029,7 @@
         <v>11</v>
       </c>
       <c r="E80" s="2">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F80" s="3" t="s">
         <v>12</v>
@@ -5055,7 +5055,7 @@
         <v>11</v>
       </c>
       <c r="E81" s="4">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F81" s="3" t="s">
         <v>12</v>
@@ -5081,7 +5081,7 @@
         <v>11</v>
       </c>
       <c r="E82" s="2">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F82" s="3" t="s">
         <v>12</v>
@@ -5107,7 +5107,7 @@
         <v>11</v>
       </c>
       <c r="E83" s="4">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F83" s="3" t="s">
         <v>12</v>
@@ -5133,7 +5133,7 @@
         <v>11</v>
       </c>
       <c r="E84" s="2">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F84" s="3" t="s">
         <v>12</v>
@@ -5159,7 +5159,7 @@
         <v>11</v>
       </c>
       <c r="E85" s="4">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F85" s="3" t="s">
         <v>12</v>
@@ -5185,7 +5185,7 @@
         <v>11</v>
       </c>
       <c r="E86" s="2">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F86" s="3" t="s">
         <v>12</v>
@@ -5211,7 +5211,7 @@
         <v>11</v>
       </c>
       <c r="E87" s="4">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F87" s="3" t="s">
         <v>12</v>
@@ -5237,7 +5237,7 @@
         <v>11</v>
       </c>
       <c r="E88" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F88" s="3" t="s">
         <v>12</v>
@@ -5263,7 +5263,7 @@
         <v>11</v>
       </c>
       <c r="E89" s="4">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F89" s="3" t="s">
         <v>12</v>
@@ -5289,7 +5289,7 @@
         <v>11</v>
       </c>
       <c r="E90" s="2">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="F90" s="3" t="s">
         <v>12</v>
@@ -5315,7 +5315,7 @@
         <v>11</v>
       </c>
       <c r="E91" s="4">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F91" s="3" t="s">
         <v>12</v>
@@ -5341,7 +5341,7 @@
         <v>11</v>
       </c>
       <c r="E92" s="2">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F92" s="3" t="s">
         <v>12</v>
@@ -5367,7 +5367,7 @@
         <v>11</v>
       </c>
       <c r="E93" s="4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F93" s="3" t="s">
         <v>12</v>
@@ -5393,7 +5393,7 @@
         <v>11</v>
       </c>
       <c r="E94" s="2">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F94" s="3" t="s">
         <v>12</v>
@@ -5445,7 +5445,7 @@
         <v>11</v>
       </c>
       <c r="E96" s="2">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F96" s="3" t="s">
         <v>12</v>
@@ -5471,7 +5471,7 @@
         <v>11</v>
       </c>
       <c r="E97" s="4">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F97" s="3" t="s">
         <v>12</v>
@@ -5497,7 +5497,7 @@
         <v>11</v>
       </c>
       <c r="E98" s="2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F98" s="3" t="s">
         <v>12</v>
@@ -5523,7 +5523,7 @@
         <v>11</v>
       </c>
       <c r="E99" s="4">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F99" s="3" t="s">
         <v>12</v>
@@ -5549,7 +5549,7 @@
         <v>11</v>
       </c>
       <c r="E100" s="2">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F100" s="3" t="s">
         <v>12</v>
@@ -5575,7 +5575,7 @@
         <v>11</v>
       </c>
       <c r="E101" s="4">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F101" s="3" t="s">
         <v>12</v>
@@ -5601,7 +5601,7 @@
         <v>11</v>
       </c>
       <c r="E102" s="2">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F102" s="3" t="s">
         <v>12</v>
@@ -5627,7 +5627,7 @@
         <v>11</v>
       </c>
       <c r="E103" s="4">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F103" s="3" t="s">
         <v>12</v>
@@ -5653,7 +5653,7 @@
         <v>11</v>
       </c>
       <c r="E104" s="2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F104" s="3" t="s">
         <v>12</v>
@@ -5679,7 +5679,7 @@
         <v>11</v>
       </c>
       <c r="E105" s="4">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F105" s="3" t="s">
         <v>12</v>
@@ -5705,7 +5705,7 @@
         <v>11</v>
       </c>
       <c r="E106" s="2">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F106" s="3" t="s">
         <v>12</v>
@@ -5731,7 +5731,7 @@
         <v>11</v>
       </c>
       <c r="E107" s="4">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F107" s="3" t="s">
         <v>12</v>
@@ -5757,7 +5757,7 @@
         <v>11</v>
       </c>
       <c r="E108" s="2">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F108" s="3" t="s">
         <v>12</v>
@@ -5783,7 +5783,7 @@
         <v>11</v>
       </c>
       <c r="E109" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="F109" s="3" t="s">
         <v>12</v>
@@ -5809,7 +5809,7 @@
         <v>11</v>
       </c>
       <c r="E110" s="2">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="F110" s="3" t="s">
         <v>12</v>
@@ -5835,7 +5835,7 @@
         <v>11</v>
       </c>
       <c r="E111" s="4">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F111" s="3" t="s">
         <v>12</v>
@@ -5861,7 +5861,7 @@
         <v>11</v>
       </c>
       <c r="E112" s="2">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F112" s="3" t="s">
         <v>12</v>
@@ -5887,7 +5887,7 @@
         <v>11</v>
       </c>
       <c r="E113" s="4">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F113" s="3" t="s">
         <v>12</v>
@@ -5913,7 +5913,7 @@
         <v>11</v>
       </c>
       <c r="E114" s="2">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F114" s="3" t="s">
         <v>12</v>
@@ -5939,7 +5939,7 @@
         <v>11</v>
       </c>
       <c r="E115" s="4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F115" s="3" t="s">
         <v>12</v>
@@ -5965,7 +5965,7 @@
         <v>11</v>
       </c>
       <c r="E116" s="2">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F116" s="3" t="s">
         <v>12</v>
@@ -5991,7 +5991,7 @@
         <v>11</v>
       </c>
       <c r="E117" s="4">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F117" s="3" t="s">
         <v>12</v>
@@ -6017,7 +6017,7 @@
         <v>11</v>
       </c>
       <c r="E118" s="2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F118" s="3" t="s">
         <v>12</v>
@@ -6043,7 +6043,7 @@
         <v>11</v>
       </c>
       <c r="E119" s="4">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F119" s="3" t="s">
         <v>12</v>
@@ -6069,7 +6069,7 @@
         <v>11</v>
       </c>
       <c r="E120" s="2">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F120" s="3" t="s">
         <v>12</v>
@@ -6095,7 +6095,7 @@
         <v>11</v>
       </c>
       <c r="E121" s="4">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F121" s="3" t="s">
         <v>12</v>
@@ -6121,7 +6121,7 @@
         <v>11</v>
       </c>
       <c r="E122" s="2">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F122" s="3" t="s">
         <v>12</v>
@@ -6147,7 +6147,7 @@
         <v>11</v>
       </c>
       <c r="E123" s="4">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F123" s="3" t="s">
         <v>12</v>
@@ -6173,7 +6173,7 @@
         <v>11</v>
       </c>
       <c r="E124" s="2">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F124" s="3" t="s">
         <v>12</v>
@@ -6199,7 +6199,7 @@
         <v>11</v>
       </c>
       <c r="E125" s="4">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F125" s="3" t="s">
         <v>12</v>
@@ -6251,7 +6251,7 @@
         <v>11</v>
       </c>
       <c r="E127" s="4">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F127" s="3" t="s">
         <v>12</v>
@@ -6277,7 +6277,7 @@
         <v>11</v>
       </c>
       <c r="E128" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F128" s="3" t="s">
         <v>12</v>
@@ -6329,7 +6329,7 @@
         <v>11</v>
       </c>
       <c r="E130" s="2">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F130" s="3" t="s">
         <v>12</v>
@@ -6355,7 +6355,7 @@
         <v>11</v>
       </c>
       <c r="E131" s="4">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F131" s="3" t="s">
         <v>12</v>
@@ -6381,7 +6381,7 @@
         <v>11</v>
       </c>
       <c r="E132" s="2">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F132" s="3" t="s">
         <v>12</v>
@@ -6407,7 +6407,7 @@
         <v>11</v>
       </c>
       <c r="E133" s="4">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F133" s="3" t="s">
         <v>12</v>
@@ -6433,7 +6433,7 @@
         <v>11</v>
       </c>
       <c r="E134" s="2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F134" s="3" t="s">
         <v>12</v>
@@ -6459,7 +6459,7 @@
         <v>11</v>
       </c>
       <c r="E135" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F135" s="3" t="s">
         <v>12</v>
@@ -6485,7 +6485,7 @@
         <v>11</v>
       </c>
       <c r="E136" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F136" s="3" t="s">
         <v>12</v>
@@ -6511,7 +6511,7 @@
         <v>11</v>
       </c>
       <c r="E137" s="4">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F137" s="3" t="s">
         <v>12</v>
@@ -6537,7 +6537,7 @@
         <v>11</v>
       </c>
       <c r="E138" s="2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F138" s="3" t="s">
         <v>12</v>
@@ -6563,7 +6563,7 @@
         <v>11</v>
       </c>
       <c r="E139" s="4">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F139" s="3" t="s">
         <v>12</v>
@@ -6589,7 +6589,7 @@
         <v>11</v>
       </c>
       <c r="E140" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F140" s="3" t="s">
         <v>12</v>
@@ -6615,7 +6615,7 @@
         <v>11</v>
       </c>
       <c r="E141" s="4">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F141" s="3" t="s">
         <v>12</v>
@@ -6641,7 +6641,7 @@
         <v>11</v>
       </c>
       <c r="E142" s="2">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F142" s="3" t="s">
         <v>12</v>
@@ -6667,7 +6667,7 @@
         <v>11</v>
       </c>
       <c r="E143" s="4">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F143" s="3" t="s">
         <v>12</v>
@@ -6693,7 +6693,7 @@
         <v>11</v>
       </c>
       <c r="E144" s="2">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F144" s="3" t="s">
         <v>12</v>
@@ -6719,7 +6719,7 @@
         <v>11</v>
       </c>
       <c r="E145" s="4">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F145" s="3" t="s">
         <v>12</v>
@@ -6745,7 +6745,7 @@
         <v>11</v>
       </c>
       <c r="E146" s="2">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F146" s="3" t="s">
         <v>12</v>
@@ -6771,7 +6771,7 @@
         <v>11</v>
       </c>
       <c r="E147" s="4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F147" s="3" t="s">
         <v>12</v>
@@ -6797,7 +6797,7 @@
         <v>11</v>
       </c>
       <c r="E148" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F148" s="3" t="s">
         <v>12</v>
@@ -6823,7 +6823,7 @@
         <v>11</v>
       </c>
       <c r="E149" s="4">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F149" s="3" t="s">
         <v>12</v>
@@ -6849,7 +6849,7 @@
         <v>11</v>
       </c>
       <c r="E150" s="2">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F150" s="3" t="s">
         <v>12</v>
@@ -6875,7 +6875,7 @@
         <v>11</v>
       </c>
       <c r="E151" s="4">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F151" s="3" t="s">
         <v>12</v>
@@ -6901,7 +6901,7 @@
         <v>11</v>
       </c>
       <c r="E152" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F152" s="3" t="s">
         <v>12</v>
@@ -6927,7 +6927,7 @@
         <v>11</v>
       </c>
       <c r="E153" s="4">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F153" s="3" t="s">
         <v>12</v>
@@ -6953,7 +6953,7 @@
         <v>11</v>
       </c>
       <c r="E154" s="2">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F154" s="3" t="s">
         <v>12</v>
@@ -6979,7 +6979,7 @@
         <v>11</v>
       </c>
       <c r="E155" s="4">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F155" s="3" t="s">
         <v>12</v>
@@ -7005,7 +7005,7 @@
         <v>11</v>
       </c>
       <c r="E156" s="2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F156" s="3" t="s">
         <v>12</v>
@@ -7031,7 +7031,7 @@
         <v>11</v>
       </c>
       <c r="E157" s="4">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F157" s="3" t="s">
         <v>12</v>
@@ -7057,7 +7057,7 @@
         <v>11</v>
       </c>
       <c r="E158" s="2">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F158" s="3" t="s">
         <v>12</v>
@@ -7083,7 +7083,7 @@
         <v>11</v>
       </c>
       <c r="E159" s="4">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F159" s="3" t="s">
         <v>12</v>
@@ -7109,7 +7109,7 @@
         <v>11</v>
       </c>
       <c r="E160" s="2">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="F160" s="3" t="s">
         <v>12</v>
@@ -7135,7 +7135,7 @@
         <v>11</v>
       </c>
       <c r="E161" s="4">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F161" s="3" t="s">
         <v>12</v>
@@ -7187,7 +7187,7 @@
         <v>11</v>
       </c>
       <c r="E163" s="4">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F163" s="3" t="s">
         <v>12</v>
@@ -7213,7 +7213,7 @@
         <v>11</v>
       </c>
       <c r="E164" s="2">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F164" s="3" t="s">
         <v>12</v>
@@ -7239,7 +7239,7 @@
         <v>11</v>
       </c>
       <c r="E165" s="4">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F165" s="3" t="s">
         <v>12</v>
@@ -7265,7 +7265,7 @@
         <v>11</v>
       </c>
       <c r="E166" s="2">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F166" s="3" t="s">
         <v>12</v>
@@ -7291,7 +7291,7 @@
         <v>11</v>
       </c>
       <c r="E167" s="4">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F167" s="3" t="s">
         <v>12</v>
@@ -7317,7 +7317,7 @@
         <v>11</v>
       </c>
       <c r="E168" s="2">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F168" s="3" t="s">
         <v>12</v>
@@ -7343,7 +7343,7 @@
         <v>11</v>
       </c>
       <c r="E169" s="4">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F169" s="3" t="s">
         <v>12</v>
@@ -7369,7 +7369,7 @@
         <v>11</v>
       </c>
       <c r="E170" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F170" s="3" t="s">
         <v>12</v>
@@ -7395,7 +7395,7 @@
         <v>11</v>
       </c>
       <c r="E171" s="4">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F171" s="3" t="s">
         <v>12</v>
@@ -7421,7 +7421,7 @@
         <v>11</v>
       </c>
       <c r="E172" s="2">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F172" s="3" t="s">
         <v>12</v>
@@ -7473,7 +7473,7 @@
         <v>11</v>
       </c>
       <c r="E174" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F174" s="3" t="s">
         <v>12</v>
@@ -7499,7 +7499,7 @@
         <v>11</v>
       </c>
       <c r="E175" s="4">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="F175" s="3" t="s">
         <v>12</v>
@@ -7525,7 +7525,7 @@
         <v>11</v>
       </c>
       <c r="E176" s="2">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F176" s="3" t="s">
         <v>12</v>
@@ -7577,7 +7577,7 @@
         <v>11</v>
       </c>
       <c r="E178" s="2">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F178" s="3" t="s">
         <v>12</v>
@@ -7603,7 +7603,7 @@
         <v>11</v>
       </c>
       <c r="E179" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F179" s="3" t="s">
         <v>12</v>
@@ -7629,7 +7629,7 @@
         <v>11</v>
       </c>
       <c r="E180" s="2">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F180" s="3" t="s">
         <v>12</v>
@@ -7655,7 +7655,7 @@
         <v>11</v>
       </c>
       <c r="E181" s="4">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F181" s="3" t="s">
         <v>12</v>
@@ -7681,7 +7681,7 @@
         <v>11</v>
       </c>
       <c r="E182" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F182" s="3" t="s">
         <v>12</v>
@@ -7707,7 +7707,7 @@
         <v>11</v>
       </c>
       <c r="E183" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="F183" s="3" t="s">
         <v>12</v>
@@ -7733,7 +7733,7 @@
         <v>11</v>
       </c>
       <c r="E184" s="2">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F184" s="3" t="s">
         <v>12</v>
@@ -7759,7 +7759,7 @@
         <v>11</v>
       </c>
       <c r="E185" s="4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F185" s="3" t="s">
         <v>12</v>
@@ -7785,7 +7785,7 @@
         <v>11</v>
       </c>
       <c r="E186" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F186" s="3" t="s">
         <v>12</v>
@@ -7811,7 +7811,7 @@
         <v>11</v>
       </c>
       <c r="E187" s="4">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F187" s="3" t="s">
         <v>12</v>
@@ -7837,7 +7837,7 @@
         <v>11</v>
       </c>
       <c r="E188" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F188" s="3" t="s">
         <v>12</v>
@@ -7863,7 +7863,7 @@
         <v>11</v>
       </c>
       <c r="E189" s="4">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="F189" s="3" t="s">
         <v>12</v>
@@ -7889,7 +7889,7 @@
         <v>11</v>
       </c>
       <c r="E190" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F190" s="3" t="s">
         <v>12</v>
@@ -7915,7 +7915,7 @@
         <v>11</v>
       </c>
       <c r="E191" s="4">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F191" s="3" t="s">
         <v>12</v>
@@ -7941,7 +7941,7 @@
         <v>11</v>
       </c>
       <c r="E192" s="2">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F192" s="3" t="s">
         <v>12</v>
@@ -7967,7 +7967,7 @@
         <v>11</v>
       </c>
       <c r="E193" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F193" s="3" t="s">
         <v>12</v>
@@ -7993,7 +7993,7 @@
         <v>11</v>
       </c>
       <c r="E194" s="2">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F194" s="3" t="s">
         <v>12</v>
@@ -8019,7 +8019,7 @@
         <v>11</v>
       </c>
       <c r="E195" s="4">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F195" s="3" t="s">
         <v>12</v>
@@ -8045,7 +8045,7 @@
         <v>11</v>
       </c>
       <c r="E196" s="2">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F196" s="3" t="s">
         <v>12</v>
@@ -8071,7 +8071,7 @@
         <v>11</v>
       </c>
       <c r="E197" s="4">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F197" s="3" t="s">
         <v>12</v>
@@ -8097,7 +8097,7 @@
         <v>11</v>
       </c>
       <c r="E198" s="2">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F198" s="3" t="s">
         <v>12</v>
@@ -8123,7 +8123,7 @@
         <v>11</v>
       </c>
       <c r="E199" s="4">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F199" s="3" t="s">
         <v>12</v>
@@ -8149,7 +8149,7 @@
         <v>11</v>
       </c>
       <c r="E200" s="2">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F200" s="3" t="s">
         <v>12</v>
@@ -8175,7 +8175,7 @@
         <v>11</v>
       </c>
       <c r="E201" s="4">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F201" s="3" t="s">
         <v>12</v>
@@ -8201,7 +8201,7 @@
         <v>11</v>
       </c>
       <c r="E202" s="2">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F202" s="3" t="s">
         <v>12</v>
@@ -8227,7 +8227,7 @@
         <v>11</v>
       </c>
       <c r="E203" s="4">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F203" s="3" t="s">
         <v>12</v>
@@ -8253,7 +8253,7 @@
         <v>11</v>
       </c>
       <c r="E204" s="2">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F204" s="3" t="s">
         <v>12</v>
@@ -8279,7 +8279,7 @@
         <v>11</v>
       </c>
       <c r="E205" s="4">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F205" s="3" t="s">
         <v>12</v>
@@ -8331,7 +8331,7 @@
         <v>11</v>
       </c>
       <c r="E207" s="4">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F207" s="3" t="s">
         <v>12</v>
@@ -8357,7 +8357,7 @@
         <v>11</v>
       </c>
       <c r="E208" s="2">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F208" s="3" t="s">
         <v>12</v>
@@ -8383,7 +8383,7 @@
         <v>11</v>
       </c>
       <c r="E209" s="4">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F209" s="3" t="s">
         <v>12</v>
@@ -8409,7 +8409,7 @@
         <v>11</v>
       </c>
       <c r="E210" s="2">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F210" s="3" t="s">
         <v>12</v>
@@ -8435,7 +8435,7 @@
         <v>11</v>
       </c>
       <c r="E211" s="4">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F211" s="3" t="s">
         <v>12</v>
@@ -8461,7 +8461,7 @@
         <v>11</v>
       </c>
       <c r="E212" s="2">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F212" s="3" t="s">
         <v>12</v>
@@ -8513,7 +8513,7 @@
         <v>11</v>
       </c>
       <c r="E214" s="2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F214" s="3" t="s">
         <v>12</v>
@@ -8539,7 +8539,7 @@
         <v>11</v>
       </c>
       <c r="E215" s="4">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F215" s="3" t="s">
         <v>12</v>
@@ -8565,7 +8565,7 @@
         <v>11</v>
       </c>
       <c r="E216" s="2">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F216" s="3" t="s">
         <v>12</v>
@@ -8591,7 +8591,7 @@
         <v>11</v>
       </c>
       <c r="E217" s="4">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F217" s="3" t="s">
         <v>12</v>
@@ -8617,7 +8617,7 @@
         <v>11</v>
       </c>
       <c r="E218" s="2">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F218" s="3" t="s">
         <v>12</v>
@@ -8643,7 +8643,7 @@
         <v>11</v>
       </c>
       <c r="E219" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F219" s="3" t="s">
         <v>12</v>
@@ -8669,7 +8669,7 @@
         <v>11</v>
       </c>
       <c r="E220" s="2">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="F220" s="3" t="s">
         <v>12</v>
@@ -8695,7 +8695,7 @@
         <v>11</v>
       </c>
       <c r="E221" s="4">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="F221" s="3" t="s">
         <v>12</v>
@@ -8721,7 +8721,7 @@
         <v>11</v>
       </c>
       <c r="E222" s="2">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F222" s="3" t="s">
         <v>12</v>
@@ -8747,7 +8747,7 @@
         <v>11</v>
       </c>
       <c r="E223" s="4">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F223" s="3" t="s">
         <v>12</v>
@@ -8773,7 +8773,7 @@
         <v>11</v>
       </c>
       <c r="E224" s="2">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F224" s="3" t="s">
         <v>12</v>
@@ -8799,7 +8799,7 @@
         <v>11</v>
       </c>
       <c r="E225" s="4">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F225" s="3" t="s">
         <v>12</v>
@@ -8825,7 +8825,7 @@
         <v>11</v>
       </c>
       <c r="E226" s="2">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F226" s="3" t="s">
         <v>12</v>
@@ -8851,7 +8851,7 @@
         <v>11</v>
       </c>
       <c r="E227" s="4">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F227" s="3" t="s">
         <v>12</v>
@@ -8877,7 +8877,7 @@
         <v>11</v>
       </c>
       <c r="E228" s="2">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F228" s="3" t="s">
         <v>12</v>
@@ -8903,7 +8903,7 @@
         <v>11</v>
       </c>
       <c r="E229" s="4">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F229" s="3" t="s">
         <v>12</v>
@@ -8929,7 +8929,7 @@
         <v>11</v>
       </c>
       <c r="E230" s="2">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F230" s="3" t="s">
         <v>12</v>
@@ -8955,7 +8955,7 @@
         <v>11</v>
       </c>
       <c r="E231" s="4">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F231" s="3" t="s">
         <v>12</v>
@@ -8981,7 +8981,7 @@
         <v>11</v>
       </c>
       <c r="E232" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F232" s="3" t="s">
         <v>12</v>
@@ -9007,7 +9007,7 @@
         <v>11</v>
       </c>
       <c r="E233" s="4">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F233" s="3" t="s">
         <v>12</v>
@@ -9033,7 +9033,7 @@
         <v>11</v>
       </c>
       <c r="E234" s="2">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F234" s="3" t="s">
         <v>12</v>
@@ -9059,7 +9059,7 @@
         <v>11</v>
       </c>
       <c r="E235" s="4">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F235" s="3" t="s">
         <v>12</v>
@@ -9085,7 +9085,7 @@
         <v>11</v>
       </c>
       <c r="E236" s="2">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F236" s="3" t="s">
         <v>12</v>
@@ -9111,7 +9111,7 @@
         <v>11</v>
       </c>
       <c r="E237" s="4">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F237" s="3" t="s">
         <v>12</v>
@@ -9137,7 +9137,7 @@
         <v>11</v>
       </c>
       <c r="E238" s="2">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F238" s="3" t="s">
         <v>12</v>
@@ -9163,7 +9163,7 @@
         <v>11</v>
       </c>
       <c r="E239" s="4">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F239" s="3" t="s">
         <v>12</v>
@@ -9189,7 +9189,7 @@
         <v>11</v>
       </c>
       <c r="E240" s="2">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F240" s="3" t="s">
         <v>12</v>
@@ -9215,7 +9215,7 @@
         <v>11</v>
       </c>
       <c r="E241" s="4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F241" s="3" t="s">
         <v>12</v>
@@ -9241,7 +9241,7 @@
         <v>11</v>
       </c>
       <c r="E242" s="2">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F242" s="3" t="s">
         <v>12</v>
@@ -9267,7 +9267,7 @@
         <v>11</v>
       </c>
       <c r="E243" s="4">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F243" s="3" t="s">
         <v>12</v>
@@ -9293,7 +9293,7 @@
         <v>11</v>
       </c>
       <c r="E244" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F244" s="3" t="s">
         <v>12</v>
@@ -9319,7 +9319,7 @@
         <v>11</v>
       </c>
       <c r="E245" s="4">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F245" s="3" t="s">
         <v>12</v>
@@ -9345,7 +9345,7 @@
         <v>11</v>
       </c>
       <c r="E246" s="2">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F246" s="3" t="s">
         <v>12</v>
@@ -9371,7 +9371,7 @@
         <v>11</v>
       </c>
       <c r="E247" s="4">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F247" s="3" t="s">
         <v>12</v>
@@ -9397,7 +9397,7 @@
         <v>11</v>
       </c>
       <c r="E248" s="2">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F248" s="3" t="s">
         <v>12</v>
@@ -9423,7 +9423,7 @@
         <v>11</v>
       </c>
       <c r="E249" s="4">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F249" s="3" t="s">
         <v>12</v>
@@ -9449,7 +9449,7 @@
         <v>11</v>
       </c>
       <c r="E250" s="2">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F250" s="3" t="s">
         <v>12</v>
@@ -9475,7 +9475,7 @@
         <v>11</v>
       </c>
       <c r="E251" s="4">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F251" s="3" t="s">
         <v>12</v>
@@ -9501,7 +9501,7 @@
         <v>11</v>
       </c>
       <c r="E252" s="2">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F252" s="3" t="s">
         <v>12</v>
@@ -9527,7 +9527,7 @@
         <v>11</v>
       </c>
       <c r="E253" s="4">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F253" s="3" t="s">
         <v>12</v>
@@ -9553,7 +9553,7 @@
         <v>11</v>
       </c>
       <c r="E254" s="2">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F254" s="3" t="s">
         <v>12</v>
@@ -9579,7 +9579,7 @@
         <v>11</v>
       </c>
       <c r="E255" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F255" s="3" t="s">
         <v>12</v>
@@ -9605,7 +9605,7 @@
         <v>11</v>
       </c>
       <c r="E256" s="2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F256" s="3" t="s">
         <v>12</v>
@@ -9631,7 +9631,7 @@
         <v>11</v>
       </c>
       <c r="E257" s="4">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F257" s="3" t="s">
         <v>12</v>
@@ -9657,7 +9657,7 @@
         <v>11</v>
       </c>
       <c r="E258" s="2">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F258" s="3" t="s">
         <v>12</v>
@@ -9683,7 +9683,7 @@
         <v>11</v>
       </c>
       <c r="E259" s="4">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F259" s="3" t="s">
         <v>12</v>
@@ -9709,7 +9709,7 @@
         <v>11</v>
       </c>
       <c r="E260" s="2">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F260" s="3" t="s">
         <v>12</v>
@@ -9735,7 +9735,7 @@
         <v>11</v>
       </c>
       <c r="E261" s="4">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F261" s="3" t="s">
         <v>12</v>
@@ -9761,7 +9761,7 @@
         <v>11</v>
       </c>
       <c r="E262" s="2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F262" s="3" t="s">
         <v>12</v>
@@ -9787,7 +9787,7 @@
         <v>11</v>
       </c>
       <c r="E263" s="4">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F263" s="3" t="s">
         <v>12</v>
@@ -9813,7 +9813,7 @@
         <v>11</v>
       </c>
       <c r="E264" s="2">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F264" s="3" t="s">
         <v>12</v>
@@ -9839,7 +9839,7 @@
         <v>11</v>
       </c>
       <c r="E265" s="4">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F265" s="3" t="s">
         <v>12</v>
@@ -9865,7 +9865,7 @@
         <v>11</v>
       </c>
       <c r="E266" s="2">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F266" s="3" t="s">
         <v>12</v>
@@ -9891,7 +9891,7 @@
         <v>11</v>
       </c>
       <c r="E267" s="4">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F267" s="3" t="s">
         <v>12</v>
@@ -9917,7 +9917,7 @@
         <v>11</v>
       </c>
       <c r="E268" s="2">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F268" s="3" t="s">
         <v>12</v>
@@ -9943,7 +9943,7 @@
         <v>11</v>
       </c>
       <c r="E269" s="4">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F269" s="3" t="s">
         <v>12</v>
@@ -9969,7 +9969,7 @@
         <v>11</v>
       </c>
       <c r="E270" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F270" s="3" t="s">
         <v>12</v>
@@ -9995,7 +9995,7 @@
         <v>11</v>
       </c>
       <c r="E271" s="4">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F271" s="3" t="s">
         <v>12</v>
@@ -10021,7 +10021,7 @@
         <v>11</v>
       </c>
       <c r="E272" s="2">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F272" s="3" t="s">
         <v>12</v>
@@ -10047,7 +10047,7 @@
         <v>11</v>
       </c>
       <c r="E273" s="4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F273" s="3" t="s">
         <v>12</v>
@@ -10073,7 +10073,7 @@
         <v>11</v>
       </c>
       <c r="E274" s="2">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F274" s="3" t="s">
         <v>12</v>
@@ -10099,7 +10099,7 @@
         <v>11</v>
       </c>
       <c r="E275" s="4">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F275" s="3" t="s">
         <v>12</v>
@@ -10125,7 +10125,7 @@
         <v>11</v>
       </c>
       <c r="E276" s="2">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F276" s="3" t="s">
         <v>12</v>
@@ -10151,7 +10151,7 @@
         <v>11</v>
       </c>
       <c r="E277" s="4">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F277" s="3" t="s">
         <v>12</v>
@@ -10177,7 +10177,7 @@
         <v>11</v>
       </c>
       <c r="E278" s="2">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F278" s="3" t="s">
         <v>12</v>
@@ -10203,7 +10203,7 @@
         <v>11</v>
       </c>
       <c r="E279" s="4">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F279" s="3" t="s">
         <v>12</v>
@@ -10229,7 +10229,7 @@
         <v>11</v>
       </c>
       <c r="E280" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F280" s="3" t="s">
         <v>12</v>
@@ -10255,7 +10255,7 @@
         <v>11</v>
       </c>
       <c r="E281" s="4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F281" s="3" t="s">
         <v>12</v>
@@ -10281,7 +10281,7 @@
         <v>11</v>
       </c>
       <c r="E282" s="2">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F282" s="3" t="s">
         <v>12</v>
@@ -10307,7 +10307,7 @@
         <v>11</v>
       </c>
       <c r="E283" s="4">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F283" s="3" t="s">
         <v>12</v>
@@ -10333,7 +10333,7 @@
         <v>11</v>
       </c>
       <c r="E284" s="2">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F284" s="3" t="s">
         <v>12</v>
@@ -10359,7 +10359,7 @@
         <v>11</v>
       </c>
       <c r="E285" s="4">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F285" s="3" t="s">
         <v>12</v>
@@ -10385,7 +10385,7 @@
         <v>11</v>
       </c>
       <c r="E286" s="2">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F286" s="3" t="s">
         <v>12</v>
@@ -10411,7 +10411,7 @@
         <v>11</v>
       </c>
       <c r="E287" s="4">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F287" s="3" t="s">
         <v>12</v>
@@ -10437,7 +10437,7 @@
         <v>11</v>
       </c>
       <c r="E288" s="2">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F288" s="3" t="s">
         <v>12</v>
@@ -10463,7 +10463,7 @@
         <v>11</v>
       </c>
       <c r="E289" s="4">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F289" s="3" t="s">
         <v>12</v>
@@ -10489,7 +10489,7 @@
         <v>11</v>
       </c>
       <c r="E290" s="2">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="F290" s="3" t="s">
         <v>12</v>
@@ -10515,7 +10515,7 @@
         <v>11</v>
       </c>
       <c r="E291" s="4">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F291" s="3" t="s">
         <v>12</v>
@@ -10541,7 +10541,7 @@
         <v>11</v>
       </c>
       <c r="E292" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F292" s="3" t="s">
         <v>12</v>
@@ -10567,7 +10567,7 @@
         <v>11</v>
       </c>
       <c r="E293" s="4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F293" s="3" t="s">
         <v>12</v>
@@ -10593,7 +10593,7 @@
         <v>11</v>
       </c>
       <c r="E294" s="2">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F294" s="3" t="s">
         <v>12</v>
@@ -10619,7 +10619,7 @@
         <v>11</v>
       </c>
       <c r="E295" s="4">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F295" s="3" t="s">
         <v>12</v>
@@ -10645,7 +10645,7 @@
         <v>11</v>
       </c>
       <c r="E296" s="2">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F296" s="3" t="s">
         <v>12</v>
@@ -10671,7 +10671,7 @@
         <v>11</v>
       </c>
       <c r="E297" s="4">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F297" s="3" t="s">
         <v>12</v>
@@ -10697,7 +10697,7 @@
         <v>11</v>
       </c>
       <c r="E298" s="2">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F298" s="3" t="s">
         <v>12</v>
@@ -10723,7 +10723,7 @@
         <v>11</v>
       </c>
       <c r="E299" s="4">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F299" s="3" t="s">
         <v>12</v>
@@ -10749,7 +10749,7 @@
         <v>11</v>
       </c>
       <c r="E300" s="2">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F300" s="3" t="s">
         <v>12</v>
@@ -10775,7 +10775,7 @@
         <v>11</v>
       </c>
       <c r="E301" s="4">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F301" s="3" t="s">
         <v>12</v>
@@ -10801,7 +10801,7 @@
         <v>11</v>
       </c>
       <c r="E302" s="2">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F302" s="3" t="s">
         <v>12</v>
@@ -10827,7 +10827,7 @@
         <v>11</v>
       </c>
       <c r="E303" s="4">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="F303" s="3" t="s">
         <v>12</v>
@@ -10853,7 +10853,7 @@
         <v>11</v>
       </c>
       <c r="E304" s="2">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F304" s="3" t="s">
         <v>12</v>
@@ -10905,7 +10905,7 @@
         <v>11</v>
       </c>
       <c r="E306" s="2">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F306" s="3" t="s">
         <v>12</v>
@@ -10931,7 +10931,7 @@
         <v>11</v>
       </c>
       <c r="E307" s="4">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F307" s="3" t="s">
         <v>12</v>
@@ -10957,7 +10957,7 @@
         <v>11</v>
       </c>
       <c r="E308" s="2">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F308" s="3" t="s">
         <v>12</v>
@@ -10983,7 +10983,7 @@
         <v>11</v>
       </c>
       <c r="E309" s="4">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F309" s="3" t="s">
         <v>12</v>
@@ -11009,7 +11009,7 @@
         <v>11</v>
       </c>
       <c r="E310" s="2">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F310" s="3" t="s">
         <v>12</v>
@@ -11035,7 +11035,7 @@
         <v>11</v>
       </c>
       <c r="E311" s="4">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F311" s="3" t="s">
         <v>12</v>
@@ -11061,7 +11061,7 @@
         <v>11</v>
       </c>
       <c r="E312" s="2">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F312" s="3" t="s">
         <v>12</v>
@@ -11087,7 +11087,7 @@
         <v>11</v>
       </c>
       <c r="E313" s="4">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F313" s="3" t="s">
         <v>12</v>
@@ -11113,7 +11113,7 @@
         <v>11</v>
       </c>
       <c r="E314" s="2">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F314" s="3" t="s">
         <v>12</v>
@@ -11139,7 +11139,7 @@
         <v>11</v>
       </c>
       <c r="E315" s="4">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F315" s="3" t="s">
         <v>12</v>
@@ -11165,7 +11165,7 @@
         <v>11</v>
       </c>
       <c r="E316" s="2">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F316" s="3" t="s">
         <v>12</v>
@@ -11191,7 +11191,7 @@
         <v>11</v>
       </c>
       <c r="E317" s="4">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F317" s="3" t="s">
         <v>12</v>
@@ -11217,7 +11217,7 @@
         <v>11</v>
       </c>
       <c r="E318" s="2">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F318" s="3" t="s">
         <v>12</v>
@@ -11243,7 +11243,7 @@
         <v>11</v>
       </c>
       <c r="E319" s="4">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F319" s="3" t="s">
         <v>12</v>
@@ -11269,7 +11269,7 @@
         <v>11</v>
       </c>
       <c r="E320" s="2">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F320" s="3" t="s">
         <v>12</v>
@@ -11295,7 +11295,7 @@
         <v>11</v>
       </c>
       <c r="E321" s="4">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F321" s="3" t="s">
         <v>12</v>
@@ -11321,7 +11321,7 @@
         <v>11</v>
       </c>
       <c r="E322" s="2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F322" s="3" t="s">
         <v>12</v>
@@ -11347,7 +11347,7 @@
         <v>11</v>
       </c>
       <c r="E323" s="4">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F323" s="3" t="s">
         <v>12</v>
@@ -11373,7 +11373,7 @@
         <v>11</v>
       </c>
       <c r="E324" s="2">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F324" s="3" t="s">
         <v>12</v>
@@ -11399,7 +11399,7 @@
         <v>11</v>
       </c>
       <c r="E325" s="4">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F325" s="3" t="s">
         <v>12</v>
@@ -11425,7 +11425,7 @@
         <v>11</v>
       </c>
       <c r="E326" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F326" s="3" t="s">
         <v>12</v>
@@ -11451,7 +11451,7 @@
         <v>11</v>
       </c>
       <c r="E327" s="4">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F327" s="3" t="s">
         <v>12</v>
@@ -11477,7 +11477,7 @@
         <v>11</v>
       </c>
       <c r="E328" s="2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F328" s="3" t="s">
         <v>12</v>
@@ -11503,7 +11503,7 @@
         <v>11</v>
       </c>
       <c r="E329" s="4">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F329" s="3" t="s">
         <v>12</v>
@@ -11529,7 +11529,7 @@
         <v>11</v>
       </c>
       <c r="E330" s="2">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F330" s="3" t="s">
         <v>12</v>
@@ -11555,7 +11555,7 @@
         <v>11</v>
       </c>
       <c r="E331" s="4">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F331" s="3" t="s">
         <v>12</v>
@@ -11581,7 +11581,7 @@
         <v>11</v>
       </c>
       <c r="E332" s="2">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F332" s="3" t="s">
         <v>12</v>
@@ -11607,7 +11607,7 @@
         <v>11</v>
       </c>
       <c r="E333" s="4">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F333" s="3" t="s">
         <v>12</v>
@@ -11633,7 +11633,7 @@
         <v>11</v>
       </c>
       <c r="E334" s="2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F334" s="3" t="s">
         <v>12</v>
@@ -11659,7 +11659,7 @@
         <v>11</v>
       </c>
       <c r="E335" s="4">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F335" s="3" t="s">
         <v>12</v>
@@ -11685,7 +11685,7 @@
         <v>11</v>
       </c>
       <c r="E336" s="2">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F336" s="3" t="s">
         <v>12</v>
@@ -11711,7 +11711,7 @@
         <v>11</v>
       </c>
       <c r="E337" s="4">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="F337" s="3" t="s">
         <v>12</v>
@@ -11737,7 +11737,7 @@
         <v>11</v>
       </c>
       <c r="E338" s="2">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F338" s="3" t="s">
         <v>12</v>
@@ -11763,7 +11763,7 @@
         <v>11</v>
       </c>
       <c r="E339" s="4">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F339" s="3" t="s">
         <v>12</v>
@@ -11789,7 +11789,7 @@
         <v>11</v>
       </c>
       <c r="E340" s="2">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F340" s="3" t="s">
         <v>12</v>
@@ -11815,7 +11815,7 @@
         <v>11</v>
       </c>
       <c r="E341" s="4">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F341" s="3" t="s">
         <v>12</v>
@@ -11841,7 +11841,7 @@
         <v>11</v>
       </c>
       <c r="E342" s="2">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="F342" s="3" t="s">
         <v>12</v>
@@ -11867,7 +11867,7 @@
         <v>11</v>
       </c>
       <c r="E343" s="4">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F343" s="3" t="s">
         <v>12</v>
@@ -11893,7 +11893,7 @@
         <v>11</v>
       </c>
       <c r="E344" s="2">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F344" s="3" t="s">
         <v>12</v>
@@ -11919,7 +11919,7 @@
         <v>11</v>
       </c>
       <c r="E345" s="4">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F345" s="3" t="s">
         <v>12</v>
@@ -11945,7 +11945,7 @@
         <v>11</v>
       </c>
       <c r="E346" s="2">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F346" s="3" t="s">
         <v>12</v>
@@ -11971,7 +11971,7 @@
         <v>11</v>
       </c>
       <c r="E347" s="4">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F347" s="3" t="s">
         <v>12</v>
@@ -11997,7 +11997,7 @@
         <v>11</v>
       </c>
       <c r="E348" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F348" s="3" t="s">
         <v>12</v>
@@ -12075,7 +12075,7 @@
         <v>11</v>
       </c>
       <c r="E351" s="4">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F351" s="3" t="s">
         <v>12</v>
@@ -12101,7 +12101,7 @@
         <v>11</v>
       </c>
       <c r="E352" s="2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F352" s="3" t="s">
         <v>12</v>
@@ -12127,7 +12127,7 @@
         <v>11</v>
       </c>
       <c r="E353" s="4">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="F353" s="3" t="s">
         <v>12</v>
@@ -12179,7 +12179,7 @@
         <v>11</v>
       </c>
       <c r="E355" s="4">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F355" s="3" t="s">
         <v>12</v>
@@ -12205,7 +12205,7 @@
         <v>11</v>
       </c>
       <c r="E356" s="2">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F356" s="3" t="s">
         <v>12</v>
@@ -12231,7 +12231,7 @@
         <v>11</v>
       </c>
       <c r="E357" s="4">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F357" s="3" t="s">
         <v>12</v>
@@ -12257,7 +12257,7 @@
         <v>11</v>
       </c>
       <c r="E358" s="2">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F358" s="3" t="s">
         <v>12</v>
@@ -12283,7 +12283,7 @@
         <v>11</v>
       </c>
       <c r="E359" s="4">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F359" s="3" t="s">
         <v>12</v>
@@ -12309,7 +12309,7 @@
         <v>11</v>
       </c>
       <c r="E360" s="2">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F360" s="3" t="s">
         <v>12</v>
@@ -12361,7 +12361,7 @@
         <v>11</v>
       </c>
       <c r="E362" s="2">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F362" s="3" t="s">
         <v>12</v>
@@ -12387,7 +12387,7 @@
         <v>11</v>
       </c>
       <c r="E363" s="4">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="F363" s="3" t="s">
         <v>12</v>
@@ -12413,7 +12413,7 @@
         <v>11</v>
       </c>
       <c r="E364" s="2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F364" s="3" t="s">
         <v>12</v>
@@ -12439,7 +12439,7 @@
         <v>11</v>
       </c>
       <c r="E365" s="4">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F365" s="3" t="s">
         <v>12</v>
@@ -12465,7 +12465,7 @@
         <v>11</v>
       </c>
       <c r="E366" s="2">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="F366" s="3" t="s">
         <v>12</v>
@@ -12491,7 +12491,7 @@
         <v>11</v>
       </c>
       <c r="E367" s="4">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F367" s="3" t="s">
         <v>12</v>
@@ -12517,7 +12517,7 @@
         <v>11</v>
       </c>
       <c r="E368" s="2">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F368" s="3" t="s">
         <v>12</v>
@@ -12543,7 +12543,7 @@
         <v>11</v>
       </c>
       <c r="E369" s="4">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F369" s="3" t="s">
         <v>12</v>
@@ -12569,7 +12569,7 @@
         <v>11</v>
       </c>
       <c r="E370" s="2">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="F370" s="3" t="s">
         <v>12</v>
@@ -12595,7 +12595,7 @@
         <v>11</v>
       </c>
       <c r="E371" s="4">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F371" s="3" t="s">
         <v>12</v>
@@ -12621,7 +12621,7 @@
         <v>11</v>
       </c>
       <c r="E372" s="2">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F372" s="3" t="s">
         <v>12</v>
@@ -12647,7 +12647,7 @@
         <v>11</v>
       </c>
       <c r="E373" s="4">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F373" s="3" t="s">
         <v>12</v>
@@ -12673,7 +12673,7 @@
         <v>11</v>
       </c>
       <c r="E374" s="2">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F374" s="3" t="s">
         <v>12</v>
@@ -12699,7 +12699,7 @@
         <v>11</v>
       </c>
       <c r="E375" s="4">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F375" s="3" t="s">
         <v>12</v>
@@ -12725,7 +12725,7 @@
         <v>11</v>
       </c>
       <c r="E376" s="2">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F376" s="3" t="s">
         <v>12</v>
@@ -12751,7 +12751,7 @@
         <v>11</v>
       </c>
       <c r="E377" s="4">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F377" s="3" t="s">
         <v>12</v>
@@ -12777,7 +12777,7 @@
         <v>11</v>
       </c>
       <c r="E378" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F378" s="3" t="s">
         <v>12</v>
@@ -12803,7 +12803,7 @@
         <v>11</v>
       </c>
       <c r="E379" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F379" s="3" t="s">
         <v>12</v>
@@ -12829,7 +12829,7 @@
         <v>11</v>
       </c>
       <c r="E380" s="2">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="F380" s="3" t="s">
         <v>12</v>
@@ -12855,7 +12855,7 @@
         <v>11</v>
       </c>
       <c r="E381" s="4">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F381" s="3" t="s">
         <v>12</v>
@@ -12881,7 +12881,7 @@
         <v>11</v>
       </c>
       <c r="E382" s="2">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F382" s="3" t="s">
         <v>12</v>
@@ -12907,7 +12907,7 @@
         <v>11</v>
       </c>
       <c r="E383" s="4">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F383" s="3" t="s">
         <v>12</v>
@@ -12959,7 +12959,7 @@
         <v>11</v>
       </c>
       <c r="E385" s="4">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F385" s="3" t="s">
         <v>12</v>
@@ -12985,7 +12985,7 @@
         <v>11</v>
       </c>
       <c r="E386" s="2">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F386" s="3" t="s">
         <v>12</v>
@@ -13011,7 +13011,7 @@
         <v>11</v>
       </c>
       <c r="E387" s="4">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F387" s="3" t="s">
         <v>12</v>
@@ -13037,7 +13037,7 @@
         <v>11</v>
       </c>
       <c r="E388" s="2">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F388" s="3" t="s">
         <v>12</v>
@@ -13063,7 +13063,7 @@
         <v>11</v>
       </c>
       <c r="E389" s="4">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="F389" s="3" t="s">
         <v>12</v>
@@ -13089,7 +13089,7 @@
         <v>11</v>
       </c>
       <c r="E390" s="2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F390" s="3" t="s">
         <v>12</v>
@@ -13115,7 +13115,7 @@
         <v>11</v>
       </c>
       <c r="E391" s="4">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F391" s="3" t="s">
         <v>12</v>
@@ -13141,7 +13141,7 @@
         <v>11</v>
       </c>
       <c r="E392" s="2">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F392" s="3" t="s">
         <v>12</v>
@@ -13167,7 +13167,7 @@
         <v>11</v>
       </c>
       <c r="E393" s="4">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F393" s="3" t="s">
         <v>12</v>
@@ -13193,7 +13193,7 @@
         <v>11</v>
       </c>
       <c r="E394" s="2">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F394" s="3" t="s">
         <v>12</v>
@@ -13219,7 +13219,7 @@
         <v>11</v>
       </c>
       <c r="E395" s="4">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F395" s="3" t="s">
         <v>12</v>
@@ -13245,7 +13245,7 @@
         <v>11</v>
       </c>
       <c r="E396" s="2">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F396" s="3" t="s">
         <v>12</v>
@@ -13271,7 +13271,7 @@
         <v>11</v>
       </c>
       <c r="E397" s="4">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F397" s="3" t="s">
         <v>12</v>
@@ -13297,7 +13297,7 @@
         <v>11</v>
       </c>
       <c r="E398" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F398" s="3" t="s">
         <v>12</v>
@@ -13323,7 +13323,7 @@
         <v>11</v>
       </c>
       <c r="E399" s="4">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F399" s="3" t="s">
         <v>12</v>
@@ -13349,7 +13349,7 @@
         <v>11</v>
       </c>
       <c r="E400" s="2">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F400" s="3" t="s">
         <v>12</v>
@@ -13375,7 +13375,7 @@
         <v>11</v>
       </c>
       <c r="E401" s="4">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="F401" s="3" t="s">
         <v>12</v>

</xml_diff>